<commit_message>
Calculatiemodel v2: aantallen uit tekeningen en NvI 21-09 verwerkt
Installatie-aantallen geteld op E.001, L.0.01-A/B, D.0.01-A/B, T.0.01,
T.0.02, R.0.01 en R.-1.01. Nieuwe tabbladen NvI en Tellingen; extra
risico's en optimalisaties naar aanleiding van de Nota van Inlichtingen.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01DGWo8ViGGiHX3nPEze7SXS
</commit_message>
<xml_diff>
--- a/calculatie/Thebe22_calculatiemodel_VDL.xlsx
+++ b/calculatie/Thebe22_calculatiemodel_VDL.xlsx
@@ -13,9 +13,11 @@
     <sheet name="Risicos" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Eenheidsprijzen" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Optimalisaties" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="NvI" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Tellingen" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Begroting'!$A$1:$K$105</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Begroting'!$A$1:$K$107</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -127,7 +129,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -193,6 +195,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -691,7 +696,7 @@
     <row r="17">
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Ook de hoeveelheden zijn aannames uit de teksten van BBN en Winkelman. Tekeningen (bijlage 1 t/m 4, L.0.01, T.0.01, R.0.01) waren bij het opstellen niet beschikbaar. Tel alle aantallen na op tekening.</t>
+          <t>Versie 2 (25-09-2026): installatie-aantallen zijn geteld op de tekeningen E.001, L.0.01-A/B, D.0.01-A/B, T.0.01, T.0.02, R.0.01 en R.-1.01 (zie tabblad 'Tellingen'). De Nota van Inlichtingen van 21-09-2026 is verwerkt (zie tabblad 'NvI'). De bouwkundige tekeningen (BBN bijlage 1 t/m 4) ontbreken nog: wandlengtes en vloeroppervlakken zijn afgeleid uit het stramien van 7,2 m. Tel alles na op DWG.</t>
         </is>
       </c>
     </row>
@@ -844,11 +849,11 @@
       </c>
       <c r="C5" s="11" t="n"/>
       <c r="D5" s="12">
-        <f>SUMIFS(Begroting!$H$2:$H$105,Begroting!$A$2:$A$105,13)</f>
+        <f>SUMIFS(Begroting!$H$2:$H$107,Begroting!$A$2:$A$107,13)</f>
         <v/>
       </c>
       <c r="E5" s="12">
-        <f>SUMIFS(Risicos!$I$2:$I$11,Risicos!$H$2:$H$11,13)</f>
+        <f>SUMIFS(Risicos!$I$2:$I$13,Risicos!$H$2:$H$13,13)</f>
         <v/>
       </c>
       <c r="F5" s="13">
@@ -873,11 +878,11 @@
       </c>
       <c r="C6" s="11" t="n"/>
       <c r="D6" s="12">
-        <f>SUMIFS(Begroting!$H$2:$H$105,Begroting!$A$2:$A$105,14)</f>
+        <f>SUMIFS(Begroting!$H$2:$H$107,Begroting!$A$2:$A$107,14)</f>
         <v/>
       </c>
       <c r="E6" s="12">
-        <f>SUMIFS(Risicos!$I$2:$I$11,Risicos!$H$2:$H$11,14)</f>
+        <f>SUMIFS(Risicos!$I$2:$I$13,Risicos!$H$2:$H$13,14)</f>
         <v/>
       </c>
       <c r="F6" s="13">
@@ -902,11 +907,11 @@
       </c>
       <c r="C7" s="11" t="n"/>
       <c r="D7" s="12">
-        <f>SUMIFS(Begroting!$H$2:$H$105,Begroting!$A$2:$A$105,15)</f>
+        <f>SUMIFS(Begroting!$H$2:$H$107,Begroting!$A$2:$A$107,15)</f>
         <v/>
       </c>
       <c r="E7" s="12">
-        <f>SUMIFS(Risicos!$I$2:$I$11,Risicos!$H$2:$H$11,15)</f>
+        <f>SUMIFS(Risicos!$I$2:$I$13,Risicos!$H$2:$H$13,15)</f>
         <v/>
       </c>
       <c r="F7" s="13">
@@ -931,11 +936,11 @@
       </c>
       <c r="C8" s="11" t="n"/>
       <c r="D8" s="12">
-        <f>SUMIFS(Begroting!$H$2:$H$105,Begroting!$A$2:$A$105,16)</f>
+        <f>SUMIFS(Begroting!$H$2:$H$107,Begroting!$A$2:$A$107,16)</f>
         <v/>
       </c>
       <c r="E8" s="12">
-        <f>SUMIFS(Risicos!$I$2:$I$11,Risicos!$H$2:$H$11,16)</f>
+        <f>SUMIFS(Risicos!$I$2:$I$13,Risicos!$H$2:$H$13,16)</f>
         <v/>
       </c>
       <c r="F8" s="13">
@@ -960,11 +965,11 @@
       </c>
       <c r="C9" s="11" t="n"/>
       <c r="D9" s="12">
-        <f>SUMIFS(Begroting!$H$2:$H$105,Begroting!$A$2:$A$105,17)</f>
+        <f>SUMIFS(Begroting!$H$2:$H$107,Begroting!$A$2:$A$107,17)</f>
         <v/>
       </c>
       <c r="E9" s="12">
-        <f>SUMIFS(Risicos!$I$2:$I$11,Risicos!$H$2:$H$11,17)</f>
+        <f>SUMIFS(Risicos!$I$2:$I$13,Risicos!$H$2:$H$13,17)</f>
         <v/>
       </c>
       <c r="F9" s="13">
@@ -989,11 +994,11 @@
       </c>
       <c r="C10" s="11" t="n"/>
       <c r="D10" s="12">
-        <f>SUMIFS(Begroting!$H$2:$H$105,Begroting!$A$2:$A$105,18)</f>
+        <f>SUMIFS(Begroting!$H$2:$H$107,Begroting!$A$2:$A$107,18)</f>
         <v/>
       </c>
       <c r="E10" s="12">
-        <f>SUMIFS(Risicos!$I$2:$I$11,Risicos!$H$2:$H$11,18)</f>
+        <f>SUMIFS(Risicos!$I$2:$I$13,Risicos!$H$2:$H$13,18)</f>
         <v/>
       </c>
       <c r="F10" s="13">
@@ -1018,11 +1023,11 @@
       </c>
       <c r="C11" s="11" t="n"/>
       <c r="D11" s="12">
-        <f>SUMIFS(Begroting!$H$2:$H$105,Begroting!$A$2:$A$105,19)</f>
+        <f>SUMIFS(Begroting!$H$2:$H$107,Begroting!$A$2:$A$107,19)</f>
         <v/>
       </c>
       <c r="E11" s="12">
-        <f>SUMIFS(Risicos!$I$2:$I$11,Risicos!$H$2:$H$11,19)</f>
+        <f>SUMIFS(Risicos!$I$2:$I$13,Risicos!$H$2:$H$13,19)</f>
         <v/>
       </c>
       <c r="F11" s="13">
@@ -1047,11 +1052,11 @@
       </c>
       <c r="C12" s="11" t="n"/>
       <c r="D12" s="12">
-        <f>SUMIFS(Begroting!$H$2:$H$105,Begroting!$A$2:$A$105,20)</f>
+        <f>SUMIFS(Begroting!$H$2:$H$107,Begroting!$A$2:$A$107,20)</f>
         <v/>
       </c>
       <c r="E12" s="12">
-        <f>SUMIFS(Risicos!$I$2:$I$11,Risicos!$H$2:$H$11,20)</f>
+        <f>SUMIFS(Risicos!$I$2:$I$13,Risicos!$H$2:$H$13,20)</f>
         <v/>
       </c>
       <c r="F12" s="13">
@@ -1076,11 +1081,11 @@
       </c>
       <c r="C13" s="11" t="n"/>
       <c r="D13" s="12">
-        <f>SUMIFS(Begroting!$H$2:$H$105,Begroting!$A$2:$A$105,21)</f>
+        <f>SUMIFS(Begroting!$H$2:$H$107,Begroting!$A$2:$A$107,21)</f>
         <v/>
       </c>
       <c r="E13" s="12">
-        <f>SUMIFS(Risicos!$I$2:$I$11,Risicos!$H$2:$H$11,21)</f>
+        <f>SUMIFS(Risicos!$I$2:$I$13,Risicos!$H$2:$H$13,21)</f>
         <v/>
       </c>
       <c r="F13" s="13">
@@ -1121,11 +1126,11 @@
       </c>
       <c r="C15" s="11" t="n"/>
       <c r="D15" s="12">
-        <f>SUMIFS(Begroting!$H$2:$H$105,Begroting!$A$2:$A$105,23)</f>
+        <f>SUMIFS(Begroting!$H$2:$H$107,Begroting!$A$2:$A$107,23)</f>
         <v/>
       </c>
       <c r="E15" s="12">
-        <f>SUMIFS(Risicos!$I$2:$I$11,Risicos!$H$2:$H$11,23)</f>
+        <f>SUMIFS(Risicos!$I$2:$I$13,Risicos!$H$2:$H$13,23)</f>
         <v/>
       </c>
       <c r="F15" s="13">
@@ -1150,11 +1155,11 @@
       </c>
       <c r="C16" s="11" t="n"/>
       <c r="D16" s="12">
-        <f>SUMIFS(Begroting!$H$2:$H$105,Begroting!$A$2:$A$105,24)</f>
+        <f>SUMIFS(Begroting!$H$2:$H$107,Begroting!$A$2:$A$107,24)</f>
         <v/>
       </c>
       <c r="E16" s="12">
-        <f>SUMIFS(Risicos!$I$2:$I$11,Risicos!$H$2:$H$11,24)</f>
+        <f>SUMIFS(Risicos!$I$2:$I$13,Risicos!$H$2:$H$13,24)</f>
         <v/>
       </c>
       <c r="F16" s="13">
@@ -1179,11 +1184,11 @@
       </c>
       <c r="C17" s="11" t="n"/>
       <c r="D17" s="12">
-        <f>SUMIFS(Begroting!$H$2:$H$105,Begroting!$A$2:$A$105,25)</f>
+        <f>SUMIFS(Begroting!$H$2:$H$107,Begroting!$A$2:$A$107,25)</f>
         <v/>
       </c>
       <c r="E17" s="12">
-        <f>SUMIFS(Risicos!$I$2:$I$11,Risicos!$H$2:$H$11,25)</f>
+        <f>SUMIFS(Risicos!$I$2:$I$13,Risicos!$H$2:$H$13,25)</f>
         <v/>
       </c>
       <c r="F17" s="13">
@@ -1208,11 +1213,11 @@
       </c>
       <c r="C18" s="11" t="n"/>
       <c r="D18" s="12">
-        <f>SUMIFS(Begroting!$H$2:$H$105,Begroting!$A$2:$A$105,26)</f>
+        <f>SUMIFS(Begroting!$H$2:$H$107,Begroting!$A$2:$A$107,26)</f>
         <v/>
       </c>
       <c r="E18" s="12">
-        <f>SUMIFS(Risicos!$I$2:$I$11,Risicos!$H$2:$H$11,26)</f>
+        <f>SUMIFS(Risicos!$I$2:$I$13,Risicos!$H$2:$H$13,26)</f>
         <v/>
       </c>
       <c r="F18" s="13">
@@ -1237,11 +1242,11 @@
       </c>
       <c r="C19" s="11" t="n"/>
       <c r="D19" s="12">
-        <f>SUMIFS(Begroting!$H$2:$H$105,Begroting!$A$2:$A$105,27)</f>
+        <f>SUMIFS(Begroting!$H$2:$H$107,Begroting!$A$2:$A$107,27)</f>
         <v/>
       </c>
       <c r="E19" s="12">
-        <f>SUMIFS(Risicos!$I$2:$I$11,Risicos!$H$2:$H$11,27)</f>
+        <f>SUMIFS(Risicos!$I$2:$I$13,Risicos!$H$2:$H$13,27)</f>
         <v/>
       </c>
       <c r="F19" s="13">
@@ -1266,11 +1271,11 @@
       </c>
       <c r="C20" s="11" t="n"/>
       <c r="D20" s="12">
-        <f>SUMIFS(Begroting!$H$2:$H$105,Begroting!$A$2:$A$105,28)</f>
+        <f>SUMIFS(Begroting!$H$2:$H$107,Begroting!$A$2:$A$107,28)</f>
         <v/>
       </c>
       <c r="E20" s="12">
-        <f>SUMIFS(Risicos!$I$2:$I$11,Risicos!$H$2:$H$11,28)</f>
+        <f>SUMIFS(Risicos!$I$2:$I$13,Risicos!$H$2:$H$13,28)</f>
         <v/>
       </c>
       <c r="F20" s="13">
@@ -1295,11 +1300,11 @@
       </c>
       <c r="C21" s="11" t="n"/>
       <c r="D21" s="12">
-        <f>SUMIFS(Begroting!$H$2:$H$105,Begroting!$A$2:$A$105,29)</f>
+        <f>SUMIFS(Begroting!$H$2:$H$107,Begroting!$A$2:$A$107,29)</f>
         <v/>
       </c>
       <c r="E21" s="12">
-        <f>SUMIFS(Risicos!$I$2:$I$11,Risicos!$H$2:$H$11,29)</f>
+        <f>SUMIFS(Risicos!$I$2:$I$13,Risicos!$H$2:$H$13,29)</f>
         <v/>
       </c>
       <c r="F21" s="13">
@@ -1324,11 +1329,11 @@
       </c>
       <c r="C22" s="11" t="n"/>
       <c r="D22" s="12">
-        <f>SUMIFS(Begroting!$H$2:$H$105,Begroting!$A$2:$A$105,30)</f>
+        <f>SUMIFS(Begroting!$H$2:$H$107,Begroting!$A$2:$A$107,30)</f>
         <v/>
       </c>
       <c r="E22" s="12">
-        <f>SUMIFS(Risicos!$I$2:$I$11,Risicos!$H$2:$H$11,30)</f>
+        <f>SUMIFS(Risicos!$I$2:$I$13,Risicos!$H$2:$H$13,30)</f>
         <v/>
       </c>
       <c r="F22" s="13">
@@ -1353,11 +1358,11 @@
       </c>
       <c r="C23" s="11" t="n"/>
       <c r="D23" s="12">
-        <f>SUMIFS(Begroting!$H$2:$H$105,Begroting!$A$2:$A$105,31)</f>
+        <f>SUMIFS(Begroting!$H$2:$H$107,Begroting!$A$2:$A$107,31)</f>
         <v/>
       </c>
       <c r="E23" s="12">
-        <f>SUMIFS(Risicos!$I$2:$I$11,Risicos!$H$2:$H$11,31)</f>
+        <f>SUMIFS(Risicos!$I$2:$I$13,Risicos!$H$2:$H$13,31)</f>
         <v/>
       </c>
       <c r="F23" s="13">
@@ -1382,11 +1387,11 @@
       </c>
       <c r="C24" s="11" t="n"/>
       <c r="D24" s="12">
-        <f>SUMIFS(Begroting!$H$2:$H$105,Begroting!$A$2:$A$105,32)</f>
+        <f>SUMIFS(Begroting!$H$2:$H$107,Begroting!$A$2:$A$107,32)</f>
         <v/>
       </c>
       <c r="E24" s="12">
-        <f>SUMIFS(Risicos!$I$2:$I$11,Risicos!$H$2:$H$11,32)</f>
+        <f>SUMIFS(Risicos!$I$2:$I$13,Risicos!$H$2:$H$13,32)</f>
         <v/>
       </c>
       <c r="F24" s="13">
@@ -1411,11 +1416,11 @@
       </c>
       <c r="C25" s="11" t="n"/>
       <c r="D25" s="12">
-        <f>SUMIFS(Begroting!$H$2:$H$105,Begroting!$A$2:$A$105,33)</f>
+        <f>SUMIFS(Begroting!$H$2:$H$107,Begroting!$A$2:$A$107,33)</f>
         <v/>
       </c>
       <c r="E25" s="12">
-        <f>SUMIFS(Risicos!$I$2:$I$11,Risicos!$H$2:$H$11,33)</f>
+        <f>SUMIFS(Risicos!$I$2:$I$13,Risicos!$H$2:$H$13,33)</f>
         <v/>
       </c>
       <c r="F25" s="13">
@@ -1440,11 +1445,11 @@
       </c>
       <c r="C26" s="11" t="n"/>
       <c r="D26" s="12">
-        <f>SUMIFS(Begroting!$H$2:$H$105,Begroting!$A$2:$A$105,34)</f>
+        <f>SUMIFS(Begroting!$H$2:$H$107,Begroting!$A$2:$A$107,34)</f>
         <v/>
       </c>
       <c r="E26" s="12">
-        <f>SUMIFS(Risicos!$I$2:$I$11,Risicos!$H$2:$H$11,34)</f>
+        <f>SUMIFS(Risicos!$I$2:$I$13,Risicos!$H$2:$H$13,34)</f>
         <v/>
       </c>
       <c r="F26" s="13">
@@ -1485,11 +1490,11 @@
       </c>
       <c r="C28" s="11" t="n"/>
       <c r="D28" s="12">
-        <f>SUMIFS(Begroting!$H$2:$H$105,Begroting!$A$2:$A$105,36)</f>
+        <f>SUMIFS(Begroting!$H$2:$H$107,Begroting!$A$2:$A$107,36)</f>
         <v/>
       </c>
       <c r="E28" s="12">
-        <f>SUMIFS(Risicos!$I$2:$I$11,Risicos!$H$2:$H$11,36)</f>
+        <f>SUMIFS(Risicos!$I$2:$I$13,Risicos!$H$2:$H$13,36)</f>
         <v/>
       </c>
       <c r="F28" s="13">
@@ -1514,11 +1519,11 @@
       </c>
       <c r="C29" s="11" t="n"/>
       <c r="D29" s="12">
-        <f>SUMIFS(Begroting!$H$2:$H$105,Begroting!$A$2:$A$105,37)</f>
+        <f>SUMIFS(Begroting!$H$2:$H$107,Begroting!$A$2:$A$107,37)</f>
         <v/>
       </c>
       <c r="E29" s="12">
-        <f>SUMIFS(Risicos!$I$2:$I$11,Risicos!$H$2:$H$11,37)</f>
+        <f>SUMIFS(Risicos!$I$2:$I$13,Risicos!$H$2:$H$13,37)</f>
         <v/>
       </c>
       <c r="F29" s="13">
@@ -1543,11 +1548,11 @@
       </c>
       <c r="C30" s="11" t="n"/>
       <c r="D30" s="12">
-        <f>SUMIFS(Begroting!$H$2:$H$105,Begroting!$A$2:$A$105,38)</f>
+        <f>SUMIFS(Begroting!$H$2:$H$107,Begroting!$A$2:$A$107,38)</f>
         <v/>
       </c>
       <c r="E30" s="12">
-        <f>SUMIFS(Risicos!$I$2:$I$11,Risicos!$H$2:$H$11,38)</f>
+        <f>SUMIFS(Risicos!$I$2:$I$13,Risicos!$H$2:$H$13,38)</f>
         <v/>
       </c>
       <c r="F30" s="13">
@@ -1725,7 +1730,7 @@
         </is>
       </c>
       <c r="F44" s="21">
-        <f>Risicos!I13/F35</f>
+        <f>Risicos!I15/F35</f>
         <v/>
       </c>
     </row>
@@ -1741,7 +1746,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K107"/>
+  <dimension ref="A1:K109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1839,7 +1844,7 @@
         </is>
       </c>
       <c r="F2" s="24" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="G2" s="25" t="n">
         <v>4200</v>
@@ -1860,7 +1865,7 @@
       </c>
       <c r="K2" s="23" t="inlineStr">
         <is>
-          <t>Aantal nieuw vs. te verplaatsen uittellen op W-tekeningen; bestek zegt: uitgaan van grootste bouwgrootte</t>
+          <t>Telling L.0.01-A/B: 34 fancoils nodig (29 kamers + 3 keuken 0.24 + 1 keuken 0.64 + 1 personeelsruimte 0.73); D.0.01-A/B toont 29 bestaande → 5 nieuw. Bouwgrootte: grootste aanhouden (E&amp;W 7.4.2)</t>
         </is>
       </c>
     </row>
@@ -1889,7 +1894,7 @@
         </is>
       </c>
       <c r="F3" s="24" t="n">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="G3" s="25" t="n">
         <v>1400</v>
@@ -1910,7 +1915,7 @@
       </c>
       <c r="K3" s="23" t="inlineStr">
         <is>
-          <t>Aantal uittellen op tekening</t>
+          <t>29 bestaande fancoils volgens demontagetekeningen D.0.01-A (19) en D.0.01-B (10)</t>
         </is>
       </c>
     </row>
@@ -1989,7 +1994,7 @@
         </is>
       </c>
       <c r="F5" s="24" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="G5" s="25" t="n">
         <v>190</v>
@@ -2135,7 +2140,7 @@
         </is>
       </c>
       <c r="F8" s="24" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="G8" s="25" t="n">
         <v>220</v>
@@ -2154,7 +2159,11 @@
           <t>Richtprijs</t>
         </is>
       </c>
-      <c r="K8" s="23" t="inlineStr"/>
+      <c r="K8" s="23" t="inlineStr">
+        <is>
+          <t>34 fancoils + 6 kanaalverwarmers</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="23" t="n">
@@ -2217,12 +2226,12 @@
       </c>
       <c r="C10" s="23" t="inlineStr">
         <is>
-          <t>Douche-aansluiting warm/koud incl. afvoer (0.42, 0.70, 0.71)</t>
+          <t>Douche-aansluiting warm/koud incl. afvoer (0.37, 0.42, 0.70, 0.71)</t>
         </is>
       </c>
       <c r="D10" s="23" t="inlineStr">
         <is>
-          <t>E&amp;W 6.1/6.2</t>
+          <t>E&amp;W 6.1/6.2 + T.0.01</t>
         </is>
       </c>
       <c r="E10" s="23" t="inlineStr">
@@ -2231,7 +2240,7 @@
         </is>
       </c>
       <c r="F10" s="24" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G10" s="25" t="n">
         <v>1500</v>
@@ -2252,7 +2261,7 @@
       </c>
       <c r="K10" s="23" t="inlineStr">
         <is>
-          <t>Aantal douches uittellen op T.0.01</t>
+          <t>T.0.01: 4 douches 0.42 + 4 douches 0.37 + 2 (0.70/0.71). 0.37 staat niet in de E&amp;W-tekst</t>
         </is>
       </c>
     </row>
@@ -2281,7 +2290,7 @@
         </is>
       </c>
       <c r="F11" s="24" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G11" s="25" t="n">
         <v>1150</v>
@@ -2302,7 +2311,7 @@
       </c>
       <c r="K11" s="23" t="inlineStr">
         <is>
-          <t>Voorgeschreven fabricaat</t>
+          <t>Voorgeschreven fabricaat; 10 douches volgens T.0.01</t>
         </is>
       </c>
     </row>
@@ -2363,12 +2372,12 @@
       </c>
       <c r="C13" s="23" t="inlineStr">
         <is>
-          <t>Wastafels ruimte 0.42 incl. toestel en aansluiting</t>
+          <t>Wastafels 0.37 en 0.42 incl. toestel en aansluiting</t>
         </is>
       </c>
       <c r="D13" s="23" t="inlineStr">
         <is>
-          <t>E&amp;W 6.1/6.3</t>
+          <t>E&amp;W 6.1/6.3 + T.0.01</t>
         </is>
       </c>
       <c r="E13" s="23" t="inlineStr">
@@ -2377,7 +2386,7 @@
         </is>
       </c>
       <c r="F13" s="24" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G13" s="25" t="n">
         <v>950</v>
@@ -2398,7 +2407,7 @@
       </c>
       <c r="K13" s="23" t="inlineStr">
         <is>
-          <t>Aantal uittellen</t>
+          <t>T.0.01: 4 in 0.42 + 4 in 0.37</t>
         </is>
       </c>
     </row>
@@ -2413,12 +2422,12 @@
       </c>
       <c r="C14" s="23" t="inlineStr">
         <is>
-          <t>Aansluiten aanrechten 0.24, 0.64 en pantry 0.01 (warm/koud + afvoer; 0.24 via nieuw tracé naar vetafscheider)</t>
+          <t>Aansluiten tappunten aanrechten 0.24 (3), 0.64 (3) en pantry 0.01 (1) (warm/koud + afvoer; 0.24 via nieuw tracé naar vetafscheider)</t>
         </is>
       </c>
       <c r="D14" s="23" t="inlineStr">
         <is>
-          <t>E&amp;W 6.1.1</t>
+          <t>E&amp;W 6.1.1 + T.0.01</t>
         </is>
       </c>
       <c r="E14" s="23" t="inlineStr">
@@ -2427,10 +2436,10 @@
         </is>
       </c>
       <c r="F14" s="24" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G14" s="25" t="n">
-        <v>1300</v>
+        <v>950</v>
       </c>
       <c r="H14" s="26">
         <f>F14*G14</f>
@@ -2555,12 +2564,12 @@
       </c>
       <c r="C17" s="23" t="inlineStr">
         <is>
-          <t>Uitbreiding VWA-stelsel (PVC / Dyka Sono in plafonds), brandmanchetten</t>
+          <t>Uitbreiding VWA-stelsel: ca. 40 m PVC in plafond parkeergarage (R.-1.01) + ca. 12 vloerdoorboringen, Dyka Sono in plafonds, brandmanchetten</t>
         </is>
       </c>
       <c r="D17" s="23" t="inlineStr">
         <is>
-          <t>E&amp;W 6.1.3</t>
+          <t>E&amp;W 6.1.3 + R.-1.01/R.0.01</t>
         </is>
       </c>
       <c r="E17" s="23" t="inlineStr">
@@ -2572,7 +2581,7 @@
         <v>1</v>
       </c>
       <c r="G17" s="25" t="n">
-        <v>9500</v>
+        <v>16000</v>
       </c>
       <c r="H17" s="26">
         <f>F17*G17</f>
@@ -2588,7 +2597,11 @@
           <t>Richtprijs</t>
         </is>
       </c>
-      <c r="K17" s="23" t="inlineStr"/>
+      <c r="K17" s="23" t="inlineStr">
+        <is>
+          <t>R.-1.01: nieuwe leiding in kelder naar vetafscheider. Kernboringen door BG-vloer met vloerverwarming</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="23" t="n">
@@ -2707,7 +2720,7 @@
         </is>
       </c>
       <c r="F20" s="24" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="G20" s="25" t="n">
         <v>1350</v>
@@ -2728,7 +2741,7 @@
       </c>
       <c r="K20" s="23" t="inlineStr">
         <is>
-          <t>Kanaallengtes uittrekken op L.0.01A/B</t>
+          <t>L.0.01-A/B: 29 kamers + keukens, personeelsruimte, gespreksruimten, badruimten</t>
         </is>
       </c>
     </row>
@@ -2757,7 +2770,7 @@
         </is>
       </c>
       <c r="F21" s="24" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="G21" s="25" t="n">
         <v>780</v>
@@ -2778,7 +2791,7 @@
       </c>
       <c r="K21" s="23" t="inlineStr">
         <is>
-          <t>Type onduidelijk: FDC25 (8.4.2) vs FDC M24S (9.4) – aantal uittellen</t>
+          <t>L.0.01 + E.001: 2 per kamer (toevoer + retour) = 58, plus ca. 6 in 60-min scheidingen. Type onduidelijk: FDC25 vs FDC M24S</t>
         </is>
       </c>
     </row>
@@ -2807,7 +2820,7 @@
         </is>
       </c>
       <c r="F22" s="24" t="n">
-        <v>140</v>
+        <v>230</v>
       </c>
       <c r="G22" s="25" t="n">
         <v>175</v>
@@ -2828,7 +2841,7 @@
       </c>
       <c r="K22" s="23" t="inlineStr">
         <is>
-          <t>Aantal uittellen</t>
+          <t>L.0.01: per kamer 6 roosters (CTV, CRVM, 2× RTB, 2× RRB) = 174 + ca. 56 in keukens/overige ruimten</t>
         </is>
       </c>
     </row>
@@ -2970,7 +2983,7 @@
       </c>
       <c r="K25" s="23" t="inlineStr">
         <is>
-          <t>Offerte Techno Horeca is bijgevoegd – bedrag overnemen. Let op: BBN 3.7.2 noemt wasemschouw + wandkappen</t>
+          <t>Offerte Techno Horeca is bijgevoegd – bedrag overnemen. E.001 toont 7 AK-aansluitpunten, E&amp;W 8 kappen; BBN 3.7.2 noemt wasemschouw + wandkappen</t>
         </is>
       </c>
     </row>
@@ -3045,7 +3058,7 @@
         </is>
       </c>
       <c r="F27" s="24" t="n">
-        <v>130</v>
+        <v>215</v>
       </c>
       <c r="G27" s="25" t="n">
         <v>210</v>
@@ -3066,7 +3079,7 @@
       </c>
       <c r="K27" s="23" t="inlineStr">
         <is>
-          <t>Aantal volgt uit lichtplan</t>
+          <t>E.001: A1 60x60 (92), E1/E2 downlights (36), F (8), W (9), H hanglamp (1 per kamer); typische kamers doorgerekend naar 29</t>
         </is>
       </c>
     </row>
@@ -3086,7 +3099,7 @@
       </c>
       <c r="D28" s="23" t="inlineStr">
         <is>
-          <t>E&amp;W 10.10</t>
+          <t>E&amp;W 10.10 + E.001</t>
         </is>
       </c>
       <c r="E28" s="23" t="inlineStr">
@@ -3095,7 +3108,7 @@
         </is>
       </c>
       <c r="F28" s="24" t="n">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="G28" s="25" t="n">
         <v>265</v>
@@ -3114,7 +3127,11 @@
           <t>Richtprijs</t>
         </is>
       </c>
-      <c r="K28" s="23" t="inlineStr"/>
+      <c r="K28" s="23" t="inlineStr">
+        <is>
+          <t>E.001: 11 NV/NV1-punten getekend + pictogrammen; aantal volgt uit projectering NEN 1838</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="23" t="n">
@@ -3283,7 +3300,7 @@
         </is>
       </c>
       <c r="F32" s="24" t="n">
-        <v>160</v>
+        <v>95</v>
       </c>
       <c r="G32" s="25" t="n">
         <v>135</v>
@@ -3304,7 +3321,7 @@
       </c>
       <c r="K32" s="23" t="inlineStr">
         <is>
-          <t>Incl. punten die niet op tekening staan (10.7)</t>
+          <t>E.001: KK per kamer + keukens (~32), 3O per kamer (29), Alg. (14), WM (4), DR (3), overig. Let op: punten die niet op tekening staan, horen er ook bij (10.7)</t>
         </is>
       </c>
     </row>
@@ -3650,7 +3667,7 @@
       </c>
       <c r="D40" s="23" t="inlineStr">
         <is>
-          <t>E&amp;W 11.2</t>
+          <t>E&amp;W 11.2 + E.001</t>
         </is>
       </c>
       <c r="E40" s="23" t="inlineStr">
@@ -3659,7 +3676,7 @@
         </is>
       </c>
       <c r="F40" s="24" t="n">
-        <v>80</v>
+        <v>8</v>
       </c>
       <c r="G40" s="25" t="n">
         <v>195</v>
@@ -3680,7 +3697,7 @@
       </c>
       <c r="K40" s="23" t="inlineStr">
         <is>
-          <t>Aantal volgt uit tekening</t>
+          <t>E.001: 8 D-punten (kantoor, gespreksruimten, beveiliging)</t>
         </is>
       </c>
     </row>
@@ -3700,7 +3717,7 @@
       </c>
       <c r="D41" s="23" t="inlineStr">
         <is>
-          <t>E&amp;W 11.2</t>
+          <t>E&amp;W 11.2 + E.001</t>
         </is>
       </c>
       <c r="E41" s="23" t="inlineStr">
@@ -3709,7 +3726,7 @@
         </is>
       </c>
       <c r="F41" s="24" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="G41" s="25" t="n">
         <v>320</v>
@@ -3728,7 +3745,11 @@
           <t>Richtprijs</t>
         </is>
       </c>
-      <c r="K41" s="23" t="inlineStr"/>
+      <c r="K41" s="23" t="inlineStr">
+        <is>
+          <t>E.001: 12 Wi-Fi-punten</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="23" t="n">
@@ -3888,7 +3909,7 @@
       </c>
       <c r="D45" s="23" t="inlineStr">
         <is>
-          <t>E&amp;W 12.2.3</t>
+          <t>E&amp;W 12.2.3 + E.001</t>
         </is>
       </c>
       <c r="E45" s="23" t="inlineStr">
@@ -3897,7 +3918,7 @@
         </is>
       </c>
       <c r="F45" s="24" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G45" s="25" t="n">
         <v>230</v>
@@ -3929,12 +3950,12 @@
       </c>
       <c r="C46" s="23" t="inlineStr">
         <is>
-          <t>Handbrandmelders (in deur brandslanghaspelkast) + slow-whoops klasse B</t>
+          <t>Handbrandmelders (4) + slow-whoops / sirenesokkels klasse B (ca. 35)</t>
         </is>
       </c>
       <c r="D46" s="23" t="inlineStr">
         <is>
-          <t>E&amp;W 12.2.6/12.3</t>
+          <t>E&amp;W 12.2.6/12.3 + E.001</t>
         </is>
       </c>
       <c r="E46" s="23" t="inlineStr">
@@ -3943,10 +3964,10 @@
         </is>
       </c>
       <c r="F46" s="24" t="n">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="G46" s="25" t="n">
-        <v>260</v>
+        <v>245</v>
       </c>
       <c r="H46" s="26">
         <f>F46*G46</f>
@@ -3964,7 +3985,7 @@
       </c>
       <c r="K46" s="23" t="inlineStr">
         <is>
-          <t>Extra signaalgevers zijn niet verrekenbaar</t>
+          <t>E.001: HBM 4, SW/R-SW/MS-SW-combinaties ca. 35 na doorrekenen typische kamers. Extra signaalgevers niet verrekenbaar</t>
         </is>
       </c>
     </row>
@@ -4986,7 +5007,7 @@
       </c>
       <c r="D68" s="23" t="inlineStr">
         <is>
-          <t>BBN 3.3.1/3.3.3</t>
+          <t>BBN 3.3.1/3.3.3 + NvI vraag 6</t>
         </is>
       </c>
       <c r="E68" s="23" t="inlineStr">
@@ -5016,7 +5037,7 @@
       </c>
       <c r="K68" s="23" t="inlineStr">
         <is>
-          <t>Uitgangspunt: ca. 300 m1 × 3,3 m tot betondek – uitmeten op bijlage 1 en 4</t>
+          <t>Afgeleid uit stramien 7,2 m op L.0.01/E.001: ca. 300 m1 nieuwe wand (kamerscheidend + gangwanden) × 3,3 m. NvI vraag 6: alle kamerscheidende wanden volledig nieuw. Hoogte tot betondek nameten</t>
         </is>
       </c>
     </row>
@@ -5031,12 +5052,12 @@
       </c>
       <c r="C69" s="23" t="inlineStr">
         <is>
-          <t>Toeslag verhoogde geluidsisolatie (47 dB noord, 59 dB kantoor/spreekruimten)</t>
+          <t>Toeslag verhoogde geluidsisolatie 47 dB kamers noord (0.49–0.56, 0.74–0.76)</t>
         </is>
       </c>
       <c r="D69" s="23" t="inlineStr">
         <is>
-          <t>BBN 3.3.2/3.3.3</t>
+          <t>BBN 3.3.3</t>
         </is>
       </c>
       <c r="E69" s="23" t="inlineStr">
@@ -5045,10 +5066,10 @@
         </is>
       </c>
       <c r="F69" s="24" t="n">
-        <v>250</v>
+        <v>160</v>
       </c>
       <c r="G69" s="25" t="n">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="H69" s="26">
         <f>F69*G69</f>
@@ -5066,7 +5087,7 @@
       </c>
       <c r="K69" s="23" t="inlineStr">
         <is>
-          <t>59 dB is zwaar voor metal-stud: navragen</t>
+          <t>Ca. 48 m1 × 3,3 m</t>
         </is>
       </c>
     </row>
@@ -5081,12 +5102,12 @@
       </c>
       <c r="C70" s="23" t="inlineStr">
         <is>
-          <t>Scanbehang + sauswerk wanden (beide zijden)</t>
+          <t>Toeslag 59 dB: dubbele metal-stud frame wand 155–170 mm (kantoor/gespreksruimten 0.04, 0.05, 0.62, 0.63)</t>
         </is>
       </c>
       <c r="D70" s="23" t="inlineStr">
         <is>
-          <t>BBN 3.3.1</t>
+          <t>BBN 3.3.2 / NvI vraag 5</t>
         </is>
       </c>
       <c r="E70" s="23" t="inlineStr">
@@ -5095,10 +5116,10 @@
         </is>
       </c>
       <c r="F70" s="24" t="n">
-        <v>2000</v>
+        <v>60</v>
       </c>
       <c r="G70" s="25" t="n">
-        <v>14</v>
+        <v>115</v>
       </c>
       <c r="H70" s="26">
         <f>F70*G70</f>
@@ -5106,7 +5127,7 @@
       </c>
       <c r="I70" s="23" t="inlineStr">
         <is>
-          <t>OA schilder</t>
+          <t>VDL</t>
         </is>
       </c>
       <c r="J70" s="23" t="inlineStr">
@@ -5114,7 +5135,11 @@
           <t>Richtprijs</t>
         </is>
       </c>
-      <c r="K70" s="23" t="inlineStr"/>
+      <c r="K70" s="23" t="inlineStr">
+        <is>
+          <t>NvI vraag 5: alleen haalbaar met dubbele frames; DnT,A of Rw niet beantwoord. Ca. 18 m1 × 3,3 m</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="23" t="n">
@@ -5127,24 +5152,24 @@
       </c>
       <c r="C71" s="23" t="inlineStr">
         <is>
-          <t>Deurstel EI30 akoestisch, 40-44 mm, insteekslot, elektrische sluitplaat (voorbereid op Trigion), drangers</t>
+          <t>Scanbehang + sauswerk wanden (beide zijden)</t>
         </is>
       </c>
       <c r="D71" s="23" t="inlineStr">
         <is>
-          <t>BBN 3.4.2</t>
+          <t>BBN 3.3.1</t>
         </is>
       </c>
       <c r="E71" s="23" t="inlineStr">
         <is>
-          <t>st</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="F71" s="24" t="n">
-        <v>35</v>
+        <v>2000</v>
       </c>
       <c r="G71" s="25" t="n">
-        <v>2150</v>
+        <v>14</v>
       </c>
       <c r="H71" s="26">
         <f>F71*G71</f>
@@ -5152,19 +5177,15 @@
       </c>
       <c r="I71" s="23" t="inlineStr">
         <is>
-          <t>VDL / OA leverancier</t>
+          <t>OA schilder</t>
         </is>
       </c>
       <c r="J71" s="23" t="inlineStr">
         <is>
-          <t>Offerte aanvragen</t>
-        </is>
-      </c>
-      <c r="K71" s="23" t="inlineStr">
-        <is>
-          <t>Levertijd kritisch voor planning</t>
-        </is>
-      </c>
+          <t>Richtprijs</t>
+        </is>
+      </c>
+      <c r="K71" s="23" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="23" t="n">
@@ -5177,12 +5198,12 @@
       </c>
       <c r="C72" s="23" t="inlineStr">
         <is>
-          <t>Overige binnendeurstellen (techniek, berging, gemeenschappelijk)</t>
+          <t>Deurstel EI30 akoestisch, 40-44 mm, insteekslot, elektrische sluitplaat (voorbereid op Trigion), vrijloopdranger</t>
         </is>
       </c>
       <c r="D72" s="23" t="inlineStr">
         <is>
-          <t>BBN 3.4.1</t>
+          <t>BBN 3.4.2 + E.001</t>
         </is>
       </c>
       <c r="E72" s="23" t="inlineStr">
@@ -5191,10 +5212,10 @@
         </is>
       </c>
       <c r="F72" s="24" t="n">
-        <v>8</v>
+        <v>35</v>
       </c>
       <c r="G72" s="25" t="n">
-        <v>1250</v>
+        <v>2150</v>
       </c>
       <c r="H72" s="26">
         <f>F72*G72</f>
@@ -5202,15 +5223,19 @@
       </c>
       <c r="I72" s="23" t="inlineStr">
         <is>
-          <t>VDL</t>
+          <t>VDL / OA leverancier</t>
         </is>
       </c>
       <c r="J72" s="23" t="inlineStr">
         <is>
-          <t>Richtprijs</t>
-        </is>
-      </c>
-      <c r="K72" s="23" t="inlineStr"/>
+          <t>Offerte aanvragen</t>
+        </is>
+      </c>
+      <c r="K72" s="23" t="inlineStr">
+        <is>
+          <t>29 kamerdeuren + 6 overig. E.001 toont VLD per kamerdeur maar maar 2 ES + 3 kaartlezers: BBN (ES per deur) aangehouden als strengste eis. Levertijd kritisch</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="23" t="n">
@@ -5223,7 +5248,7 @@
       </c>
       <c r="C73" s="23" t="inlineStr">
         <is>
-          <t>Sluitplan / cilinders met moedersleutelsysteem</t>
+          <t>Overige binnendeurstellen (techniek, berging, gemeenschappelijk)</t>
         </is>
       </c>
       <c r="D73" s="23" t="inlineStr">
@@ -5237,10 +5262,10 @@
         </is>
       </c>
       <c r="F73" s="24" t="n">
-        <v>45</v>
+        <v>8</v>
       </c>
       <c r="G73" s="25" t="n">
-        <v>110</v>
+        <v>1250</v>
       </c>
       <c r="H73" s="26">
         <f>F73*G73</f>
@@ -5248,7 +5273,7 @@
       </c>
       <c r="I73" s="23" t="inlineStr">
         <is>
-          <t>OA</t>
+          <t>VDL</t>
         </is>
       </c>
       <c r="J73" s="23" t="inlineStr">
@@ -5269,7 +5294,7 @@
       </c>
       <c r="C74" s="23" t="inlineStr">
         <is>
-          <t>Kleefmagneten/openzetvoorzieningen verkeersdeuren (mechanisch deel)</t>
+          <t>Sluitplan / cilinders met moedersleutelsysteem</t>
         </is>
       </c>
       <c r="D74" s="23" t="inlineStr">
@@ -5283,10 +5308,10 @@
         </is>
       </c>
       <c r="F74" s="24" t="n">
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="G74" s="25" t="n">
-        <v>260</v>
+        <v>110</v>
       </c>
       <c r="H74" s="26">
         <f>F74*G74</f>
@@ -5294,7 +5319,7 @@
       </c>
       <c r="I74" s="23" t="inlineStr">
         <is>
-          <t>VDL</t>
+          <t>OA</t>
         </is>
       </c>
       <c r="J74" s="23" t="inlineStr">
@@ -5306,33 +5331,33 @@
     </row>
     <row r="75">
       <c r="A75" s="23" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B75" s="23" t="inlineStr">
         <is>
-          <t>Vervangen plafondafwerking</t>
+          <t>Aanpassen binnenwanden, -kozijnen en deuren</t>
         </is>
       </c>
       <c r="C75" s="23" t="inlineStr">
         <is>
-          <t>Verwijderen bestaand plafond incl. constructie</t>
+          <t>Kleefmagneten/openzetvoorzieningen verkeersdeuren (mechanisch deel)</t>
         </is>
       </c>
       <c r="D75" s="23" t="inlineStr">
         <is>
-          <t>BBN 3.5</t>
+          <t>BBN 3.4.1</t>
         </is>
       </c>
       <c r="E75" s="23" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>st</t>
         </is>
       </c>
       <c r="F75" s="24" t="n">
-        <v>1250</v>
+        <v>10</v>
       </c>
       <c r="G75" s="25" t="n">
-        <v>8</v>
+        <v>260</v>
       </c>
       <c r="H75" s="26">
         <f>F75*G75</f>
@@ -5340,7 +5365,7 @@
       </c>
       <c r="I75" s="23" t="inlineStr">
         <is>
-          <t>OA plafondmonteur</t>
+          <t>VDL</t>
         </is>
       </c>
       <c r="J75" s="23" t="inlineStr">
@@ -5361,7 +5386,7 @@
       </c>
       <c r="C76" s="23" t="inlineStr">
         <is>
-          <t>Nieuw systeemplafond 600x600 incl. inspectieluiken en aanpassingen armaturen/roosters</t>
+          <t>Verwijderen bestaand plafond incl. constructie</t>
         </is>
       </c>
       <c r="D76" s="23" t="inlineStr">
@@ -5375,10 +5400,10 @@
         </is>
       </c>
       <c r="F76" s="24" t="n">
-        <v>1200</v>
+        <v>1250</v>
       </c>
       <c r="G76" s="25" t="n">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="H76" s="26">
         <f>F76*G76</f>
@@ -5398,33 +5423,33 @@
     </row>
     <row r="77">
       <c r="A77" s="23" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B77" s="23" t="inlineStr">
         <is>
-          <t>Aanpassen zonwering</t>
+          <t>Vervangen plafondafwerking</t>
         </is>
       </c>
       <c r="C77" s="23" t="inlineStr">
         <is>
-          <t>Demonteren bestaande binnenzonwering</t>
+          <t>Nieuw systeemplafond 600x600 incl. inspectieluiken en aanpassingen armaturen/roosters</t>
         </is>
       </c>
       <c r="D77" s="23" t="inlineStr">
         <is>
-          <t>BBN 3.7.1</t>
+          <t>BBN 3.5</t>
         </is>
       </c>
       <c r="E77" s="23" t="inlineStr">
         <is>
-          <t>post</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="F77" s="24" t="n">
-        <v>1</v>
+        <v>1200</v>
       </c>
       <c r="G77" s="25" t="n">
-        <v>1500</v>
+        <v>42</v>
       </c>
       <c r="H77" s="26">
         <f>F77*G77</f>
@@ -5432,7 +5457,7 @@
       </c>
       <c r="I77" s="23" t="inlineStr">
         <is>
-          <t>VDL</t>
+          <t>OA plafondmonteur</t>
         </is>
       </c>
       <c r="J77" s="23" t="inlineStr">
@@ -5440,11 +5465,7 @@
           <t>Richtprijs</t>
         </is>
       </c>
-      <c r="K77" s="23" t="inlineStr">
-        <is>
-          <t>E&amp;W 4.1.3 zegt: pand heeft geen zonwering – navragen</t>
-        </is>
-      </c>
+      <c r="K77" s="23" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="23" t="n">
@@ -5457,7 +5478,7 @@
       </c>
       <c r="C78" s="23" t="inlineStr">
         <is>
-          <t>Verduisterende gordijnen incl. rails, gelijk aan verdiepingen</t>
+          <t>Demonteren bestaande binnenzonwering</t>
         </is>
       </c>
       <c r="D78" s="23" t="inlineStr">
@@ -5467,14 +5488,14 @@
       </c>
       <c r="E78" s="23" t="inlineStr">
         <is>
-          <t>m1</t>
+          <t>post</t>
         </is>
       </c>
       <c r="F78" s="24" t="n">
-        <v>150</v>
+        <v>1</v>
       </c>
       <c r="G78" s="25" t="n">
-        <v>95</v>
+        <v>1500</v>
       </c>
       <c r="H78" s="26">
         <f>F78*G78</f>
@@ -5482,7 +5503,7 @@
       </c>
       <c r="I78" s="23" t="inlineStr">
         <is>
-          <t>OA stoffeerder</t>
+          <t>VDL</t>
         </is>
       </c>
       <c r="J78" s="23" t="inlineStr">
@@ -5492,27 +5513,27 @@
       </c>
       <c r="K78" s="23" t="inlineStr">
         <is>
-          <t>Raamlengtes uitmeten</t>
+          <t>E&amp;W 4.1.3 zegt: pand heeft geen zonwering – navragen</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="23" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B79" s="23" t="inlineStr">
         <is>
-          <t>Realiseren vaste keukenvoorzieningen en pantry's</t>
+          <t>Aanpassen zonwering</t>
         </is>
       </c>
       <c r="C79" s="23" t="inlineStr">
         <is>
-          <t>Keukenblok woonkamer (multiplex/HPL, RVS-grepen, onderkasten)</t>
+          <t>Verduisterende gordijnen incl. rails, gelijk aan verdiepingen</t>
         </is>
       </c>
       <c r="D79" s="23" t="inlineStr">
         <is>
-          <t>BBN 3.7.2</t>
+          <t>BBN 3.7.1</t>
         </is>
       </c>
       <c r="E79" s="23" t="inlineStr">
@@ -5521,10 +5542,10 @@
         </is>
       </c>
       <c r="F79" s="24" t="n">
-        <v>10</v>
+        <v>150</v>
       </c>
       <c r="G79" s="25" t="n">
-        <v>780</v>
+        <v>95</v>
       </c>
       <c r="H79" s="26">
         <f>F79*G79</f>
@@ -5532,7 +5553,7 @@
       </c>
       <c r="I79" s="23" t="inlineStr">
         <is>
-          <t>OA keukenbouwer</t>
+          <t>OA stoffeerder</t>
         </is>
       </c>
       <c r="J79" s="23" t="inlineStr">
@@ -5540,7 +5561,11 @@
           <t>Richtprijs</t>
         </is>
       </c>
-      <c r="K79" s="23" t="inlineStr"/>
+      <c r="K79" s="23" t="inlineStr">
+        <is>
+          <t>Raamlengtes uitmeten</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="23" t="n">
@@ -5553,7 +5578,7 @@
       </c>
       <c r="C80" s="23" t="inlineStr">
         <is>
-          <t>Keukenblok eetruimte</t>
+          <t>Keukenblok woonkamer (multiplex/HPL, RVS-grepen, onderkasten)</t>
         </is>
       </c>
       <c r="D80" s="23" t="inlineStr">
@@ -5567,7 +5592,7 @@
         </is>
       </c>
       <c r="F80" s="24" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="G80" s="25" t="n">
         <v>780</v>
@@ -5599,7 +5624,7 @@
       </c>
       <c r="C81" s="23" t="inlineStr">
         <is>
-          <t>Inductiekookplaat 4-pits (4 st woonkamer, 2 st eetruimte)</t>
+          <t>Keukenblok eetruimte</t>
         </is>
       </c>
       <c r="D81" s="23" t="inlineStr">
@@ -5609,14 +5634,14 @@
       </c>
       <c r="E81" s="23" t="inlineStr">
         <is>
-          <t>st</t>
+          <t>m1</t>
         </is>
       </c>
       <c r="F81" s="24" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G81" s="25" t="n">
-        <v>950</v>
+        <v>780</v>
       </c>
       <c r="H81" s="26">
         <f>F81*G81</f>
@@ -5632,11 +5657,7 @@
           <t>Richtprijs</t>
         </is>
       </c>
-      <c r="K81" s="23" t="inlineStr">
-        <is>
-          <t>E&amp;W 10.7.6 zegt: keukenapparatuur door derden – navragen</t>
-        </is>
-      </c>
+      <c r="K81" s="23" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="23" t="n">
@@ -5649,7 +5670,7 @@
       </c>
       <c r="C82" s="23" t="inlineStr">
         <is>
-          <t>RVS spoelbak + kraan gemeenschappelijke keukens</t>
+          <t>Inductiekookplaat 4-pits (4 st woonkamer, 2 st eetruimte)</t>
         </is>
       </c>
       <c r="D82" s="23" t="inlineStr">
@@ -5663,10 +5684,10 @@
         </is>
       </c>
       <c r="F82" s="24" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G82" s="25" t="n">
-        <v>520</v>
+        <v>950</v>
       </c>
       <c r="H82" s="26">
         <f>F82*G82</f>
@@ -5682,7 +5703,11 @@
           <t>Richtprijs</t>
         </is>
       </c>
-      <c r="K82" s="23" t="inlineStr"/>
+      <c r="K82" s="23" t="inlineStr">
+        <is>
+          <t>E&amp;W 10.7.6 zegt: keukenapparatuur door derden – navragen</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="23" t="n">
@@ -5695,12 +5720,12 @@
       </c>
       <c r="C83" s="23" t="inlineStr">
         <is>
-          <t>Pantry slaapkamer (werkblad, onderkast, RVS spoelbak/kraan, nis koelkast, WCD)</t>
+          <t>RVS spoelbak + kraan gemeenschappelijke keukens</t>
         </is>
       </c>
       <c r="D83" s="23" t="inlineStr">
         <is>
-          <t>BBN 3.7.3</t>
+          <t>BBN 3.7.2</t>
         </is>
       </c>
       <c r="E83" s="23" t="inlineStr">
@@ -5709,10 +5734,10 @@
         </is>
       </c>
       <c r="F83" s="24" t="n">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="G83" s="25" t="n">
-        <v>1350</v>
+        <v>520</v>
       </c>
       <c r="H83" s="26">
         <f>F83*G83</f>
@@ -5728,41 +5753,37 @@
           <t>Richtprijs</t>
         </is>
       </c>
-      <c r="K83" s="23" t="inlineStr">
-        <is>
-          <t>Aantal volgens bijlage 1. LET OP: water/afvoer naar kamers staat NIET in E&amp;W</t>
-        </is>
-      </c>
+      <c r="K83" s="23" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="23" t="n">
+        <v>28</v>
+      </c>
+      <c r="B84" s="23" t="inlineStr">
+        <is>
+          <t>Realiseren vaste keukenvoorzieningen en pantry's</t>
+        </is>
+      </c>
+      <c r="C84" s="23" t="inlineStr">
+        <is>
+          <t>Pantry slaapkamer (werkblad, onderkast, RVS spoelbak/kraan, nis koelkast, WCD)</t>
+        </is>
+      </c>
+      <c r="D84" s="23" t="inlineStr">
+        <is>
+          <t>BBN 3.7.3</t>
+        </is>
+      </c>
+      <c r="E84" s="23" t="inlineStr">
+        <is>
+          <t>st</t>
+        </is>
+      </c>
+      <c r="F84" s="24" t="n">
         <v>29</v>
       </c>
-      <c r="B84" s="23" t="inlineStr">
-        <is>
-          <t>Realiseren douchevoorzieningen</t>
-        </is>
-      </c>
-      <c r="C84" s="23" t="inlineStr">
-        <is>
-          <t>Metal-stud douchewanden, watervaste beplating</t>
-        </is>
-      </c>
-      <c r="D84" s="23" t="inlineStr">
-        <is>
-          <t>BBN 3.3.4</t>
-        </is>
-      </c>
-      <c r="E84" s="23" t="inlineStr">
-        <is>
-          <t>m2</t>
-        </is>
-      </c>
-      <c r="F84" s="24" t="n">
-        <v>80</v>
-      </c>
       <c r="G84" s="25" t="n">
-        <v>125</v>
+        <v>1350</v>
       </c>
       <c r="H84" s="26">
         <f>F84*G84</f>
@@ -5770,7 +5791,7 @@
       </c>
       <c r="I84" s="23" t="inlineStr">
         <is>
-          <t>VDL</t>
+          <t>OA keukenbouwer</t>
         </is>
       </c>
       <c r="J84" s="23" t="inlineStr">
@@ -5778,7 +5799,11 @@
           <t>Richtprijs</t>
         </is>
       </c>
-      <c r="K84" s="23" t="inlineStr"/>
+      <c r="K84" s="23" t="inlineStr">
+        <is>
+          <t>29 kamers (kk op alle plattegronden). LET OP: T.0.01/R.0.01 tonen GEEN water/afvoer naar de kamers; BBN 3.7.3 vraagt wel RVS-spoelbak + kraan</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="23" t="n">
@@ -5791,7 +5816,7 @@
       </c>
       <c r="C85" s="23" t="inlineStr">
         <is>
-          <t>Wandtegelwerk douches incl. afdichtingssysteem</t>
+          <t>Metal-stud douchewanden, watervaste beplating</t>
         </is>
       </c>
       <c r="D85" s="23" t="inlineStr">
@@ -5805,10 +5830,10 @@
         </is>
       </c>
       <c r="F85" s="24" t="n">
-        <v>160</v>
+        <v>80</v>
       </c>
       <c r="G85" s="25" t="n">
-        <v>98</v>
+        <v>125</v>
       </c>
       <c r="H85" s="26">
         <f>F85*G85</f>
@@ -5816,7 +5841,7 @@
       </c>
       <c r="I85" s="23" t="inlineStr">
         <is>
-          <t>OA tegelzetter</t>
+          <t>VDL</t>
         </is>
       </c>
       <c r="J85" s="23" t="inlineStr">
@@ -5837,12 +5862,12 @@
       </c>
       <c r="C86" s="23" t="inlineStr">
         <is>
-          <t>Vloertegels douches, antislip, incl. afschot en afdichting</t>
+          <t>Wandtegelwerk douches incl. afdichtingssysteem</t>
         </is>
       </c>
       <c r="D86" s="23" t="inlineStr">
         <is>
-          <t>BBN 3.2.3</t>
+          <t>BBN 3.3.4</t>
         </is>
       </c>
       <c r="E86" s="23" t="inlineStr">
@@ -5851,10 +5876,10 @@
         </is>
       </c>
       <c r="F86" s="24" t="n">
-        <v>45</v>
+        <v>160</v>
       </c>
       <c r="G86" s="25" t="n">
-        <v>145</v>
+        <v>98</v>
       </c>
       <c r="H86" s="26">
         <f>F86*G86</f>
@@ -5883,24 +5908,24 @@
       </c>
       <c r="C87" s="23" t="inlineStr">
         <is>
-          <t>Trespa douchedeuren incl. beslag en profielen</t>
+          <t>Vloertegels douches, antislip, incl. afschot en afdichting</t>
         </is>
       </c>
       <c r="D87" s="23" t="inlineStr">
         <is>
-          <t>BBN 3.4.3</t>
+          <t>BBN 3.2.3</t>
         </is>
       </c>
       <c r="E87" s="23" t="inlineStr">
         <is>
-          <t>st</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="F87" s="24" t="n">
-        <v>8</v>
+        <v>45</v>
       </c>
       <c r="G87" s="25" t="n">
-        <v>680</v>
+        <v>145</v>
       </c>
       <c r="H87" s="26">
         <f>F87*G87</f>
@@ -5908,7 +5933,7 @@
       </c>
       <c r="I87" s="23" t="inlineStr">
         <is>
-          <t>VDL</t>
+          <t>OA tegelzetter</t>
         </is>
       </c>
       <c r="J87" s="23" t="inlineStr">
@@ -5920,33 +5945,33 @@
     </row>
     <row r="88">
       <c r="A88" s="23" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B88" s="23" t="inlineStr">
         <is>
-          <t>Realiseren hekwerk terrein</t>
+          <t>Realiseren douchevoorzieningen</t>
         </is>
       </c>
       <c r="C88" s="23" t="inlineStr">
         <is>
-          <t>Hekwerk ≥1 m op gemetselde muur, chemische ankers, 'zwevend' boven tegels, incl. opname</t>
+          <t>Trespa douchedeuren incl. beslag en profielen</t>
         </is>
       </c>
       <c r="D88" s="23" t="inlineStr">
         <is>
-          <t>BBN 3.8.2</t>
+          <t>BBN 3.4.3</t>
         </is>
       </c>
       <c r="E88" s="23" t="inlineStr">
         <is>
-          <t>m1</t>
+          <t>st</t>
         </is>
       </c>
       <c r="F88" s="24" t="n">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="G88" s="25" t="n">
-        <v>225</v>
+        <v>680</v>
       </c>
       <c r="H88" s="26">
         <f>F88*G88</f>
@@ -5954,7 +5979,7 @@
       </c>
       <c r="I88" s="23" t="inlineStr">
         <is>
-          <t>OA hekwerk</t>
+          <t>VDL</t>
         </is>
       </c>
       <c r="J88" s="23" t="inlineStr">
@@ -5962,41 +5987,37 @@
           <t>Richtprijs</t>
         </is>
       </c>
-      <c r="K88" s="23" t="inlineStr">
-        <is>
-          <t>Lengte uitmeten</t>
-        </is>
-      </c>
+      <c r="K88" s="23" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="23" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B89" s="23" t="inlineStr">
         <is>
-          <t>Realiseren entree's, incl. bijbehorende voorzieningen</t>
+          <t>Realiseren hekwerk terrein</t>
         </is>
       </c>
       <c r="C89" s="23" t="inlineStr">
         <is>
-          <t>Drie entrees tuinzijde met hergebruik dubbele deuren</t>
+          <t>Hekwerk ≥1 m op gemetselde muur, chemische ankers, 'zwevend' boven tegels, incl. opname</t>
         </is>
       </c>
       <c r="D89" s="23" t="inlineStr">
         <is>
-          <t>BBN 3.8.1</t>
+          <t>BBN 3.8.2</t>
         </is>
       </c>
       <c r="E89" s="23" t="inlineStr">
         <is>
-          <t>st</t>
+          <t>m1</t>
         </is>
       </c>
       <c r="F89" s="24" t="n">
-        <v>3</v>
+        <v>30</v>
       </c>
       <c r="G89" s="25" t="n">
-        <v>1500</v>
+        <v>225</v>
       </c>
       <c r="H89" s="26">
         <f>F89*G89</f>
@@ -6004,7 +6025,7 @@
       </c>
       <c r="I89" s="23" t="inlineStr">
         <is>
-          <t>VDL</t>
+          <t>OA hekwerk</t>
         </is>
       </c>
       <c r="J89" s="23" t="inlineStr">
@@ -6012,7 +6033,11 @@
           <t>Richtprijs</t>
         </is>
       </c>
-      <c r="K89" s="23" t="inlineStr"/>
+      <c r="K89" s="23" t="inlineStr">
+        <is>
+          <t>Lengte uitmeten</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="23" t="n">
@@ -6025,7 +6050,7 @@
       </c>
       <c r="C90" s="23" t="inlineStr">
         <is>
-          <t>Betontegels 1x2x0,1 m als opstap + toegankelijke helling binnen ≤3 m</t>
+          <t>Drie entrees tuinzijde met hergebruik dubbele deuren</t>
         </is>
       </c>
       <c r="D90" s="23" t="inlineStr">
@@ -6035,14 +6060,14 @@
       </c>
       <c r="E90" s="23" t="inlineStr">
         <is>
-          <t>post</t>
+          <t>st</t>
         </is>
       </c>
       <c r="F90" s="24" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G90" s="25" t="n">
-        <v>4300</v>
+        <v>1500</v>
       </c>
       <c r="H90" s="26">
         <f>F90*G90</f>
@@ -6062,33 +6087,33 @@
     </row>
     <row r="91">
       <c r="A91" s="23" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B91" s="23" t="inlineStr">
         <is>
-          <t>Realiseren fietsenstalling</t>
+          <t>Realiseren entree's, incl. bijbehorende voorzieningen</t>
         </is>
       </c>
       <c r="C91" s="23" t="inlineStr">
         <is>
-          <t>Beloopbare vloerroosters Dejo o.g. over ventilatiekuil, incl. onderconstructie, thermisch verzinkt, demontabel</t>
+          <t>Betontegels 1x2x0,1 m als opstap + toegankelijke helling binnen ≤3 m</t>
         </is>
       </c>
       <c r="D91" s="23" t="inlineStr">
         <is>
-          <t>BBN 3.8.3</t>
+          <t>BBN 3.8.1</t>
         </is>
       </c>
       <c r="E91" s="23" t="inlineStr">
         <is>
-          <t>m2</t>
+          <t>post</t>
         </is>
       </c>
       <c r="F91" s="24" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="G91" s="25" t="n">
-        <v>460</v>
+        <v>4300</v>
       </c>
       <c r="H91" s="26">
         <f>F91*G91</f>
@@ -6096,7 +6121,7 @@
       </c>
       <c r="I91" s="23" t="inlineStr">
         <is>
-          <t>OA staalbouw</t>
+          <t>VDL</t>
         </is>
       </c>
       <c r="J91" s="23" t="inlineStr">
@@ -6104,11 +6129,7 @@
           <t>Richtprijs</t>
         </is>
       </c>
-      <c r="K91" s="23" t="inlineStr">
-        <is>
-          <t>m² uitmeten; fietsenrekken niet genoemd</t>
-        </is>
-      </c>
+      <c r="K91" s="23" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="23" t="n">
@@ -6121,7 +6142,7 @@
       </c>
       <c r="C92" s="23" t="inlineStr">
         <is>
-          <t>Constructieve berekening roosters/oplegging</t>
+          <t>Beloopbare vloerroosters Dejo o.g. over ventilatiekuil, incl. onderconstructie, thermisch verzinkt, demontabel</t>
         </is>
       </c>
       <c r="D92" s="23" t="inlineStr">
@@ -6131,14 +6152,14 @@
       </c>
       <c r="E92" s="23" t="inlineStr">
         <is>
-          <t>post</t>
+          <t>m2</t>
         </is>
       </c>
       <c r="F92" s="24" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="G92" s="25" t="n">
-        <v>1500</v>
+        <v>460</v>
       </c>
       <c r="H92" s="26">
         <f>F92*G92</f>
@@ -6146,7 +6167,7 @@
       </c>
       <c r="I92" s="23" t="inlineStr">
         <is>
-          <t>Constructeur</t>
+          <t>OA staalbouw</t>
         </is>
       </c>
       <c r="J92" s="23" t="inlineStr">
@@ -6154,37 +6175,41 @@
           <t>Richtprijs</t>
         </is>
       </c>
-      <c r="K92" s="23" t="inlineStr"/>
+      <c r="K92" s="23" t="inlineStr">
+        <is>
+          <t>m² uitmeten; fietsenrekken niet genoemd</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="23" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B93" s="23" t="inlineStr">
         <is>
-          <t>Doorvoeringen inbranden voor de installaties</t>
+          <t>Realiseren fietsenstalling</t>
         </is>
       </c>
       <c r="C93" s="23" t="inlineStr">
         <is>
-          <t>Brandwerende doorvoeringen (W/E/data) incl. codering en logboek conform bovenverdiepingen (VMT Zwolle)</t>
+          <t>Constructieve berekening roosters/oplegging</t>
         </is>
       </c>
       <c r="D93" s="23" t="inlineStr">
         <is>
-          <t>BBN 3.3.1 / E&amp;W 4.6/10.5.7</t>
+          <t>BBN 3.8.3</t>
         </is>
       </c>
       <c r="E93" s="23" t="inlineStr">
         <is>
-          <t>st</t>
+          <t>post</t>
         </is>
       </c>
       <c r="F93" s="24" t="n">
-        <v>260</v>
+        <v>1</v>
       </c>
       <c r="G93" s="25" t="n">
-        <v>48</v>
+        <v>1500</v>
       </c>
       <c r="H93" s="26">
         <f>F93*G93</f>
@@ -6192,49 +6217,45 @@
       </c>
       <c r="I93" s="23" t="inlineStr">
         <is>
-          <t>VMT Brandpreventie</t>
+          <t>Constructeur</t>
         </is>
       </c>
       <c r="J93" s="23" t="inlineStr">
         <is>
-          <t>Offerte aanvragen</t>
-        </is>
-      </c>
-      <c r="K93" s="23" t="inlineStr">
-        <is>
-          <t>VMT is 'voorgesteld' – offerte opvragen; aantal inschatten met installateurs</t>
-        </is>
-      </c>
+          <t>Richtprijs</t>
+        </is>
+      </c>
+      <c r="K93" s="23" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="23" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B94" s="23" t="inlineStr">
         <is>
-          <t>Evt. andere bijkomende kosten (bouwkundig)</t>
+          <t>Doorvoeringen inbranden voor de installaties</t>
         </is>
       </c>
       <c r="C94" s="23" t="inlineStr">
         <is>
-          <t>Bescherming bestaande bouw (vloeren, lift, looproutes), nulmeting met foto's</t>
+          <t>Brandwerende doorvoeringen (W/E/data) incl. codering en logboek conform bovenverdiepingen (VMT Zwolle)</t>
         </is>
       </c>
       <c r="D94" s="23" t="inlineStr">
         <is>
-          <t>BBN 6.1</t>
+          <t>BBN 3.3.1 / E&amp;W 4.6/10.5.7</t>
         </is>
       </c>
       <c r="E94" s="23" t="inlineStr">
         <is>
-          <t>post</t>
+          <t>st</t>
         </is>
       </c>
       <c r="F94" s="24" t="n">
-        <v>1</v>
+        <v>260</v>
       </c>
       <c r="G94" s="25" t="n">
-        <v>5000</v>
+        <v>48</v>
       </c>
       <c r="H94" s="26">
         <f>F94*G94</f>
@@ -6242,15 +6263,19 @@
       </c>
       <c r="I94" s="23" t="inlineStr">
         <is>
-          <t>VDL</t>
+          <t>VMT Brandpreventie</t>
         </is>
       </c>
       <c r="J94" s="23" t="inlineStr">
         <is>
-          <t>Richtprijs</t>
-        </is>
-      </c>
-      <c r="K94" s="23" t="inlineStr"/>
+          <t>Offerte aanvragen</t>
+        </is>
+      </c>
+      <c r="K94" s="23" t="inlineStr">
+        <is>
+          <t>VMT is 'voorgesteld' – offerte opvragen; aantal inschatten met installateurs</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="23" t="n">
@@ -6263,12 +6288,12 @@
       </c>
       <c r="C95" s="23" t="inlineStr">
         <is>
-          <t>Opleveringsschoonmaak</t>
+          <t>Bescherming bestaande bouw (vloeren, lift, looproutes), nulmeting met foto's</t>
         </is>
       </c>
       <c r="D95" s="23" t="inlineStr">
         <is>
-          <t>BBN 6.2</t>
+          <t>BBN 6.1</t>
         </is>
       </c>
       <c r="E95" s="23" t="inlineStr">
@@ -6280,7 +6305,7 @@
         <v>1</v>
       </c>
       <c r="G95" s="25" t="n">
-        <v>3500</v>
+        <v>5000</v>
       </c>
       <c r="H95" s="26">
         <f>F95*G95</f>
@@ -6288,7 +6313,7 @@
       </c>
       <c r="I95" s="23" t="inlineStr">
         <is>
-          <t>OA schoonmaak</t>
+          <t>VDL</t>
         </is>
       </c>
       <c r="J95" s="23" t="inlineStr">
@@ -6300,21 +6325,21 @@
     </row>
     <row r="96">
       <c r="A96" s="23" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B96" s="23" t="inlineStr">
         <is>
-          <t>Engineering en coördinatiekosten</t>
+          <t>Evt. andere bijkomende kosten (bouwkundig)</t>
         </is>
       </c>
       <c r="C96" s="23" t="inlineStr">
         <is>
-          <t>Bouwkundige engineering, detaillering, constructeur</t>
+          <t>Opleveringsschoonmaak</t>
         </is>
       </c>
       <c r="D96" s="23" t="inlineStr">
         <is>
-          <t>BBN 4.1</t>
+          <t>BBN 6.2</t>
         </is>
       </c>
       <c r="E96" s="23" t="inlineStr">
@@ -6326,7 +6351,7 @@
         <v>1</v>
       </c>
       <c r="G96" s="25" t="n">
-        <v>12000</v>
+        <v>3500</v>
       </c>
       <c r="H96" s="26">
         <f>F96*G96</f>
@@ -6334,7 +6359,7 @@
       </c>
       <c r="I96" s="23" t="inlineStr">
         <is>
-          <t>VDL / adviseur</t>
+          <t>OA schoonmaak</t>
         </is>
       </c>
       <c r="J96" s="23" t="inlineStr">
@@ -6355,12 +6380,12 @@
       </c>
       <c r="C97" s="23" t="inlineStr">
         <is>
-          <t>Installatie-engineering: werktekeningen, VABI, tapwater-, licht-, kabelberekeningen</t>
+          <t>Bouwkundige engineering, detaillering, constructeur</t>
         </is>
       </c>
       <c r="D97" s="23" t="inlineStr">
         <is>
-          <t>E&amp;W 3.7/3.9</t>
+          <t>BBN 4.1</t>
         </is>
       </c>
       <c r="E97" s="23" t="inlineStr">
@@ -6372,7 +6397,7 @@
         <v>1</v>
       </c>
       <c r="G97" s="25" t="n">
-        <v>18000</v>
+        <v>12000</v>
       </c>
       <c r="H97" s="26">
         <f>F97*G97</f>
@@ -6380,7 +6405,7 @@
       </c>
       <c r="I97" s="23" t="inlineStr">
         <is>
-          <t>OA installateurs</t>
+          <t>VDL / adviseur</t>
         </is>
       </c>
       <c r="J97" s="23" t="inlineStr">
@@ -6388,11 +6413,7 @@
           <t>Richtprijs</t>
         </is>
       </c>
-      <c r="K97" s="23" t="inlineStr">
-        <is>
-          <t>Reken op 5 weken review-cyclus met Winkelman</t>
-        </is>
-      </c>
+      <c r="K97" s="23" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="23" t="n">
@@ -6405,12 +6426,12 @@
       </c>
       <c r="C98" s="23" t="inlineStr">
         <is>
-          <t>Projectleiding, werkvoorbereiding, coördinatie nevenaannemers (Trigion) en VGM-coördinatie</t>
+          <t>Installatie-engineering: werktekeningen, VABI, tapwater-, licht-, kabelberekeningen</t>
         </is>
       </c>
       <c r="D98" s="23" t="inlineStr">
         <is>
-          <t>BBN 3.9 / E&amp;W 3.3</t>
+          <t>E&amp;W 3.7/3.9</t>
         </is>
       </c>
       <c r="E98" s="23" t="inlineStr">
@@ -6422,7 +6443,7 @@
         <v>1</v>
       </c>
       <c r="G98" s="25" t="n">
-        <v>16000</v>
+        <v>18000</v>
       </c>
       <c r="H98" s="26">
         <f>F98*G98</f>
@@ -6430,7 +6451,7 @@
       </c>
       <c r="I98" s="23" t="inlineStr">
         <is>
-          <t>VDL</t>
+          <t>OA installateurs</t>
         </is>
       </c>
       <c r="J98" s="23" t="inlineStr">
@@ -6438,25 +6459,29 @@
           <t>Richtprijs</t>
         </is>
       </c>
-      <c r="K98" s="23" t="inlineStr"/>
+      <c r="K98" s="23" t="inlineStr">
+        <is>
+          <t>Reken op 5 weken review-cyclus met Winkelman</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="23" t="n">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B99" s="23" t="inlineStr">
         <is>
-          <t>Revisietekeningen</t>
+          <t>Engineering en coördinatiekosten</t>
         </is>
       </c>
       <c r="C99" s="23" t="inlineStr">
         <is>
-          <t>Revisietekeningen (PDF + DWG/IFC), technisch dossier, opleverdossier fysiek + digitaal</t>
+          <t>Projectleiding, werkvoorbereiding, coördinatie nevenaannemers (Trigion) en VGM-coördinatie</t>
         </is>
       </c>
       <c r="D99" s="23" t="inlineStr">
         <is>
-          <t>BBN 4.6 / E&amp;W 3.9</t>
+          <t>BBN 3.9 / E&amp;W 3.3</t>
         </is>
       </c>
       <c r="E99" s="23" t="inlineStr">
@@ -6468,7 +6493,7 @@
         <v>1</v>
       </c>
       <c r="G99" s="25" t="n">
-        <v>6500</v>
+        <v>16000</v>
       </c>
       <c r="H99" s="26">
         <f>F99*G99</f>
@@ -6476,7 +6501,7 @@
       </c>
       <c r="I99" s="23" t="inlineStr">
         <is>
-          <t>VDL + OA</t>
+          <t>VDL</t>
         </is>
       </c>
       <c r="J99" s="23" t="inlineStr">
@@ -6488,33 +6513,33 @@
     </row>
     <row r="100">
       <c r="A100" s="23" t="n">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B100" s="23" t="inlineStr">
         <is>
-          <t>Algemene Bouwplaatskosten (ABK)</t>
+          <t>Revisietekeningen</t>
         </is>
       </c>
       <c r="C100" s="23" t="inlineStr">
         <is>
-          <t>Uitvoerder (VCA-Vol, dagelijks aanwezig)</t>
+          <t>Revisietekeningen (PDF + DWG/IFC), technisch dossier, opleverdossier fysiek + digitaal</t>
         </is>
       </c>
       <c r="D100" s="23" t="inlineStr">
         <is>
-          <t>BBN 3.9</t>
+          <t>BBN 4.6 / E&amp;W 3.9</t>
         </is>
       </c>
       <c r="E100" s="23" t="inlineStr">
         <is>
-          <t>week</t>
+          <t>post</t>
         </is>
       </c>
       <c r="F100" s="24" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="G100" s="25" t="n">
-        <v>2600</v>
+        <v>6500</v>
       </c>
       <c r="H100" s="26">
         <f>F100*G100</f>
@@ -6522,7 +6547,7 @@
       </c>
       <c r="I100" s="23" t="inlineStr">
         <is>
-          <t>VDL</t>
+          <t>VDL + OA</t>
         </is>
       </c>
       <c r="J100" s="23" t="inlineStr">
@@ -6530,11 +6555,7 @@
           <t>Richtprijs</t>
         </is>
       </c>
-      <c r="K100" s="23" t="inlineStr">
-        <is>
-          <t>Doorlooptijd ca. 12 weken</t>
-        </is>
-      </c>
+      <c r="K100" s="23" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="23" t="n">
@@ -6547,24 +6568,24 @@
       </c>
       <c r="C101" s="23" t="inlineStr">
         <is>
-          <t>Inpandige schaft-, sanitaire en opslagvoorzieningen</t>
+          <t>Uitvoerder (VCA-Vol, dagelijks aanwezig)</t>
         </is>
       </c>
       <c r="D101" s="23" t="inlineStr">
         <is>
-          <t>BBN 4.3</t>
+          <t>BBN 3.9</t>
         </is>
       </c>
       <c r="E101" s="23" t="inlineStr">
         <is>
-          <t>post</t>
+          <t>week</t>
         </is>
       </c>
       <c r="F101" s="24" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="G101" s="25" t="n">
-        <v>5500</v>
+        <v>2600</v>
       </c>
       <c r="H101" s="26">
         <f>F101*G101</f>
@@ -6580,7 +6601,11 @@
           <t>Richtprijs</t>
         </is>
       </c>
-      <c r="K101" s="23" t="inlineStr"/>
+      <c r="K101" s="23" t="inlineStr">
+        <is>
+          <t>Doorlooptijd ca. 12 weken</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="23" t="n">
@@ -6593,24 +6618,24 @@
       </c>
       <c r="C102" s="23" t="inlineStr">
         <is>
-          <t>Afvalcontainers gescheiden afvoer incl. vergunning</t>
+          <t>Inpandige schaft-, sanitaire en opslagvoorzieningen</t>
         </is>
       </c>
       <c r="D102" s="23" t="inlineStr">
         <is>
-          <t>BBN 4.3/6.2</t>
+          <t>BBN 4.3</t>
         </is>
       </c>
       <c r="E102" s="23" t="inlineStr">
         <is>
-          <t>st</t>
+          <t>post</t>
         </is>
       </c>
       <c r="F102" s="24" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="G102" s="25" t="n">
-        <v>475</v>
+        <v>5500</v>
       </c>
       <c r="H102" s="26">
         <f>F102*G102</f>
@@ -6618,7 +6643,7 @@
       </c>
       <c r="I102" s="23" t="inlineStr">
         <is>
-          <t>OA afval</t>
+          <t>VDL</t>
         </is>
       </c>
       <c r="J102" s="23" t="inlineStr">
@@ -6639,24 +6664,24 @@
       </c>
       <c r="C103" s="23" t="inlineStr">
         <is>
-          <t>V&amp;G-plan uitvoeringsfase, werkplan, bouwplaatsinrichting, afzettingen</t>
+          <t>Afvalcontainers gescheiden afvoer incl. vergunning</t>
         </is>
       </c>
       <c r="D103" s="23" t="inlineStr">
         <is>
-          <t>BBN 3.9/4.3/6.3</t>
+          <t>BBN 4.3/6.2</t>
         </is>
       </c>
       <c r="E103" s="23" t="inlineStr">
         <is>
-          <t>post</t>
+          <t>st</t>
         </is>
       </c>
       <c r="F103" s="24" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="G103" s="25" t="n">
-        <v>3500</v>
+        <v>475</v>
       </c>
       <c r="H103" s="26">
         <f>F103*G103</f>
@@ -6664,7 +6689,7 @@
       </c>
       <c r="I103" s="23" t="inlineStr">
         <is>
-          <t>VDL</t>
+          <t>OA afval</t>
         </is>
       </c>
       <c r="J103" s="23" t="inlineStr">
@@ -6685,12 +6710,12 @@
       </c>
       <c r="C104" s="23" t="inlineStr">
         <is>
-          <t>Klein materieel, steigers/rolsteigers, transport</t>
+          <t>V&amp;G-plan uitvoeringsfase, werkplan, bouwplaatsinrichting, afzettingen</t>
         </is>
       </c>
       <c r="D104" s="23" t="inlineStr">
         <is>
-          <t>BBN 4.2</t>
+          <t>BBN 3.9/4.3/6.3</t>
         </is>
       </c>
       <c r="E104" s="23" t="inlineStr">
@@ -6702,7 +6727,7 @@
         <v>1</v>
       </c>
       <c r="G104" s="25" t="n">
-        <v>4500</v>
+        <v>3500</v>
       </c>
       <c r="H104" s="26">
         <f>F104*G104</f>
@@ -6731,12 +6756,12 @@
       </c>
       <c r="C105" s="23" t="inlineStr">
         <is>
-          <t>Hinderbeperking bewoond gebouw (stofschotten, geluidsarm werken, bewonerscommunicatie)</t>
+          <t>Klein materieel, steigers/rolsteigers, transport</t>
         </is>
       </c>
       <c r="D105" s="23" t="inlineStr">
         <is>
-          <t>E&amp;W 3.2 / BBN 4.4</t>
+          <t>BBN 4.2</t>
         </is>
       </c>
       <c r="E105" s="23" t="inlineStr">
@@ -6748,7 +6773,7 @@
         <v>1</v>
       </c>
       <c r="G105" s="25" t="n">
-        <v>3000</v>
+        <v>4500</v>
       </c>
       <c r="H105" s="26">
         <f>F105*G105</f>
@@ -6766,27 +6791,123 @@
       </c>
       <c r="K105" s="23" t="inlineStr"/>
     </row>
-    <row r="106"/>
+    <row r="106">
+      <c r="A106" s="23" t="n">
+        <v>38</v>
+      </c>
+      <c r="B106" s="23" t="inlineStr">
+        <is>
+          <t>Algemene Bouwplaatskosten (ABK)</t>
+        </is>
+      </c>
+      <c r="C106" s="23" t="inlineStr">
+        <is>
+          <t>Parkeerkosten (betaald parkeren, 2 voertuigen, ca. 60 werkdagen)</t>
+        </is>
+      </c>
+      <c r="D106" s="23" t="inlineStr">
+        <is>
+          <t>NvI vraag 9</t>
+        </is>
+      </c>
+      <c r="E106" s="23" t="inlineStr">
+        <is>
+          <t>dag</t>
+        </is>
+      </c>
+      <c r="F106" s="24" t="n">
+        <v>120</v>
+      </c>
+      <c r="G106" s="25" t="n">
+        <v>15</v>
+      </c>
+      <c r="H106" s="26">
+        <f>F106*G106</f>
+        <v/>
+      </c>
+      <c r="I106" s="23" t="inlineStr">
+        <is>
+          <t>VDL</t>
+        </is>
+      </c>
+      <c r="J106" s="23" t="inlineStr">
+        <is>
+          <t>Richtprijs</t>
+        </is>
+      </c>
+      <c r="K106" s="23" t="inlineStr">
+        <is>
+          <t>NvI vraag 9: betaald parkeren; regeling niet beantwoord</t>
+        </is>
+      </c>
+    </row>
     <row r="107">
-      <c r="C107" s="16" t="inlineStr">
+      <c r="A107" s="23" t="n">
+        <v>38</v>
+      </c>
+      <c r="B107" s="23" t="inlineStr">
+        <is>
+          <t>Algemene Bouwplaatskosten (ABK)</t>
+        </is>
+      </c>
+      <c r="C107" s="23" t="inlineStr">
+        <is>
+          <t>Hinderbeperking bewoond gebouw (stofschotten, geluidsarm werken, bewonerscommunicatie)</t>
+        </is>
+      </c>
+      <c r="D107" s="23" t="inlineStr">
+        <is>
+          <t>E&amp;W 3.2 / BBN 4.4</t>
+        </is>
+      </c>
+      <c r="E107" s="23" t="inlineStr">
+        <is>
+          <t>post</t>
+        </is>
+      </c>
+      <c r="F107" s="24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G107" s="25" t="n">
+        <v>3000</v>
+      </c>
+      <c r="H107" s="26">
+        <f>F107*G107</f>
+        <v/>
+      </c>
+      <c r="I107" s="23" t="inlineStr">
+        <is>
+          <t>VDL</t>
+        </is>
+      </c>
+      <c r="J107" s="23" t="inlineStr">
+        <is>
+          <t>Richtprijs</t>
+        </is>
+      </c>
+      <c r="K107" s="23" t="inlineStr"/>
+    </row>
+    <row r="108"/>
+    <row r="109">
+      <c r="C109" s="16" t="inlineStr">
         <is>
           <t>Totaal directe kosten (excl. opslagen AK/W&amp;R/CAR en risico's)</t>
         </is>
       </c>
-      <c r="H107" s="28">
-        <f>SUM(H2:H105)</f>
+      <c r="H109" s="28">
+        <f>SUM(H2:H107)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K105"/>
-  <conditionalFormatting sqref="J2:J105">
+  <autoFilter ref="A1:K107"/>
+  <conditionalFormatting sqref="J2:J107">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$J2="Richtprijs"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="J2 J3 J4 J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 J40 J41 J42 J43 J44 J45 J46 J47 J48 J49 J50 J51 J52 J53 J54 J55 J56 J57 J58 J59 J60 J61 J62 J63 J64 J65 J66 J67 J68 J69 J70 J71 J72 J73 J74 J75 J76 J77 J78 J79 J80 J81 J82 J83 J84 J85 J86 J87 J88 J89 J90 J91 J92 J93 J94 J95 J96 J97 J98 J99 J100 J101 J102 J103 J104 J105" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2 J3 J4 J5 J6 J7 J8 J9 J10 J11 J12 J13 J14 J15 J16 J17 J18 J19 J20 J21 J22 J23 J24 J25 J26 J27 J28 J29 J30 J31 J32 J33 J34 J35 J36 J37 J38 J39 J40 J41 J42 J43 J44 J45 J46 J47 J48 J49 J50 J51 J52 J53 J54 J55 J56 J57 J58 J59 J60 J61 J62 J63 J64 J65 J66 J67 J68 J69 J70 J71 J72 J73 J74 J75 J76 J77 J78 J79 J80 J81 J82 J83 J84 J85 J86 J87 J88 J89 J90 J91 J92 J93 J94 J95 J96 J97 J98 J99 J100 J101 J102 J103 J104 J105 J106 J107" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Richtprijs,Offerte aanvragen,Offerte ontvangen,Eigen norm,Stelpost (voorgeschreven)"</formula1>
     </dataValidation>
   </dataValidations>
@@ -6800,7 +6921,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J14"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -7159,19 +7280,19 @@
       </c>
       <c r="B9" s="23" t="inlineStr">
         <is>
-          <t>Versnelling om vóór eind 2026 op te leveren (overwerk, extra ploegen, kerstperiode)</t>
+          <t>Versnelling om vóór eind 2026 op te leveren: start ca. 9 nov volgens NvI vraag 8 (overwerk, extra ploegen, kerstperiode)</t>
         </is>
       </c>
       <c r="C9" s="23" t="inlineStr">
         <is>
-          <t>Offerteaanvraag / BBN 6.4</t>
+          <t>Offerteaanvraag / NvI vraag 8/15</t>
         </is>
       </c>
       <c r="D9" s="29" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="E9" s="30" t="n">
-        <v>12000</v>
+        <v>15000</v>
       </c>
       <c r="F9" s="26">
         <f>D9*E9</f>
@@ -7201,16 +7322,16 @@
       </c>
       <c r="B10" s="23" t="inlineStr">
         <is>
-          <t>Pantry's slaapkamers: water en afvoer staan niet in E&amp;W</t>
+          <t>Pantry's slaapkamers: water en afvoer staan niet in E&amp;W en niet op T.0.01/R.0.01</t>
         </is>
       </c>
       <c r="C10" s="23" t="inlineStr">
         <is>
-          <t>BBN 3.7.3 vs E&amp;W 6.1/6.2</t>
+          <t>BBN 3.7.3 vs E&amp;W 6.1/6.2 + T.0.01</t>
         </is>
       </c>
       <c r="D10" s="29" t="n">
-        <v>0.5</v>
+        <v>0.35</v>
       </c>
       <c r="E10" s="30" t="n">
         <v>25000</v>
@@ -7233,7 +7354,7 @@
       </c>
       <c r="J10" s="23" t="inlineStr">
         <is>
-          <t>Groot verschil tussen documenten. Niet meegeprijsd: aanname vastleggen, bij voorkeur via de inkoper laten bevestigen.</t>
+          <t>Tekeningen bevestigen: alleen koelkast (kk) per kamer, geen tappunt. Niet meegeprijsd; uitgangspunt vastleggen.</t>
         </is>
       </c>
     </row>
@@ -7243,19 +7364,19 @@
       </c>
       <c r="B11" s="23" t="inlineStr">
         <is>
-          <t>WKO-capaciteit / inregelen onvoldoende (nooit waterzijdig ingeregeld)</t>
+          <t>Kernboringen door BG-vloer boven parkeergarage: vloerverwarming en brandwerend dichten</t>
         </is>
       </c>
       <c r="C11" s="23" t="inlineStr">
         <is>
-          <t>E&amp;W 4.2.2/7.1</t>
+          <t>R.-1.01 / E&amp;W 6.1.1</t>
         </is>
       </c>
       <c r="D11" s="29" t="n">
-        <v>0.15</v>
+        <v>0.3</v>
       </c>
       <c r="E11" s="30" t="n">
-        <v>8000</v>
+        <v>4000</v>
       </c>
       <c r="F11" s="26">
         <f>D11*E11</f>
@@ -7263,11 +7384,11 @@
       </c>
       <c r="G11" s="31" t="inlineStr">
         <is>
-          <t>Nee</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="H11" s="31" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="I11" s="26">
         <f>IF(G11="Ja",F11,0)</f>
@@ -7275,36 +7396,120 @@
       </c>
       <c r="J11" s="23" t="inlineStr">
         <is>
+          <t>Ca. 12 doorboringen; garage is apart brandcompartiment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="23" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="23" t="inlineStr">
+        <is>
+          <t>Tellingen uit PDF-tekeningen wijken af van de werkelijke aantallen</t>
+        </is>
+      </c>
+      <c r="C12" s="23" t="inlineStr">
+        <is>
+          <t>Tekeningen E.001, L.0.01, T.0.01</t>
+        </is>
+      </c>
+      <c r="D12" s="29" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="E12" s="30" t="n">
+        <v>10000</v>
+      </c>
+      <c r="F12" s="26">
+        <f>D12*E12</f>
+        <v/>
+      </c>
+      <c r="G12" s="31" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="H12" s="31" t="n">
+        <v>36</v>
+      </c>
+      <c r="I12" s="26">
+        <f>IF(G12="Ja",F12,0)</f>
+        <v/>
+      </c>
+      <c r="J12" s="23" t="inlineStr">
+        <is>
+          <t>Tellingen zijn visueel/uit tekstlabels. Laat installateurs natellen op DWG (NvI vraag 2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="23" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="23" t="inlineStr">
+        <is>
+          <t>WKO-capaciteit / inregelen onvoldoende (nooit waterzijdig ingeregeld)</t>
+        </is>
+      </c>
+      <c r="C13" s="23" t="inlineStr">
+        <is>
+          <t>E&amp;W 4.2.2/7.1</t>
+        </is>
+      </c>
+      <c r="D13" s="29" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E13" s="30" t="n">
+        <v>8000</v>
+      </c>
+      <c r="F13" s="26">
+        <f>D13*E13</f>
+        <v/>
+      </c>
+      <c r="G13" s="31" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="H13" s="31" t="n">
+        <v>13</v>
+      </c>
+      <c r="I13" s="26">
+        <f>IF(G13="Ja",F13,0)</f>
+        <v/>
+      </c>
+      <c r="J13" s="23" t="inlineStr">
+        <is>
           <t>Het bestek stelt dat de aannemer mag uitgaan van voldoende capaciteit, dus dit risico ligt bij de opdrachtgever.</t>
         </is>
       </c>
     </row>
-    <row r="12"/>
-    <row r="13">
-      <c r="B13" s="16" t="inlineStr">
+    <row r="14"/>
+    <row r="15">
+      <c r="B15" s="16" t="inlineStr">
         <is>
           <t>Totaal meegeprijsde risico's</t>
         </is>
       </c>
-      <c r="I13" s="28">
-        <f>SUM(I2:I11)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="32" t="inlineStr">
+      <c r="I15" s="28">
+        <f>SUM(I2:I13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="32" t="inlineStr">
         <is>
           <t>Totaal verwachte waarde alle risico's (ter info)</t>
         </is>
       </c>
-      <c r="I14" s="20">
-        <f>SUM(F2:F11)</f>
+      <c r="I16" s="20">
+        <f>SUM(F2:F13)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="G2:G11" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="G2:G13" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Ja,Nee"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7549,7 +7754,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -7648,15 +7853,1034 @@
       </c>
       <c r="B7" s="35" t="inlineStr">
         <is>
+          <t>HPL-douchecabines zoals op de verdiepingen i.p.v. metal-stud + tegelwerk (NvI vraag 14)</t>
+        </is>
+      </c>
+      <c r="C7" s="36" t="n">
+        <v>-9000</v>
+      </c>
+      <c r="D7" s="35" t="inlineStr">
+        <is>
+          <t>Sneller en goedkoper; privacy blijft gewaarborgd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="B8" s="35" t="inlineStr">
+        <is>
+          <t>Marmoleum naadloos doorzetten in woonkamers i.p.v. combinatie met tapijttegels (NvI vraag 11)</t>
+        </is>
+      </c>
+      <c r="C8" s="36" t="n">
+        <v>-1500</v>
+      </c>
+      <c r="D8" s="35" t="inlineStr">
+        <is>
+          <t>Minder overgangen, beter reinigbaar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" s="35" t="inlineStr">
+        <is>
+          <t>RVS-onderkasten en -werkblad in keuken 0.24 (64 personen) (NvI vraag 12)</t>
+        </is>
+      </c>
+      <c r="C9" s="36" t="n">
+        <v>6000</v>
+      </c>
+      <c r="D9" s="35" t="inlineStr">
+        <is>
+          <t>Meerprijs, maar HPL is niet hittebestendig.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="18" t="n">
+        <v>7</v>
+      </c>
+      <c r="B10" s="35" t="inlineStr">
+        <is>
           <t>Planningsvoorstel: gefaseerde oplevering (eerst zuidvleugel, dan noord)</t>
         </is>
       </c>
-      <c r="C7" s="36" t="n">
+      <c r="C10" s="36" t="n">
         <v>0</v>
       </c>
-      <c r="D7" s="35" t="inlineStr">
+      <c r="D10" s="35" t="inlineStr">
         <is>
           <t>Geen kostenverschil, wel eerder bewoonbaar en minder planningsrisico.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="45" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Nota van Inlichtingen 21-09-2026 (TN-606498) – verwerking in het model</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="35" t="inlineStr">
+        <is>
+          <t>Let op: het document bevat alleen de vragen. De antwoorden zijn 'naar individuele vragen en antwoorden vertaald' en het componentenboek staat als bijlage op TenderNed. Download deze en controleer onderstaande aannames.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="4">
+      <c r="A4" s="33" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B4" s="33" t="inlineStr">
+        <is>
+          <t>Vraag (samengevat)</t>
+        </is>
+      </c>
+      <c r="C4" s="33" t="inlineStr">
+        <is>
+          <t>Antwoord in dit document</t>
+        </is>
+      </c>
+      <c r="D4" s="33" t="inlineStr">
+        <is>
+          <t>Verwerking in model</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="37" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="37" t="inlineStr">
+        <is>
+          <t>Materiaalboek SPIE 2022 en sanitairboek ontbreken</t>
+        </is>
+      </c>
+      <c r="C5" s="37" t="inlineStr">
+        <is>
+          <t>Componentenboek toegevoegd als bijlage (niet ontvangen)</t>
+        </is>
+      </c>
+      <c r="D5" s="37" t="inlineStr">
+        <is>
+          <t>Fabricaten conform E&amp;W aangehouden; controleren tegen componentenboek.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="37" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="37" t="inlineStr">
+        <is>
+          <t>DWG-bestanden voor revisie?</t>
+        </is>
+      </c>
+      <c r="C6" s="37" t="inlineStr">
+        <is>
+          <t>Verwezen naar afzonderlijk antwoord</t>
+        </is>
+      </c>
+      <c r="D6" s="37" t="inlineStr">
+        <is>
+          <t>Revisiepost ongewijzigd. Met DWG kunnen aantallen exact worden geteld.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="37" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="37" t="inlineStr">
+        <is>
+          <t>Afprijzen van posten die van een voorstel afhangen (lichtplan, warmteverlies, fietsenstalling)</t>
+        </is>
+      </c>
+      <c r="C7" s="37" t="inlineStr">
+        <is>
+          <t>Niet in dit document</t>
+        </is>
+      </c>
+      <c r="D7" s="37" t="inlineStr">
+        <is>
+          <t>Als vaste prijs op basis van het bestek; engineering in post E36.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="37" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="37" t="inlineStr">
+        <is>
+          <t>Stoot- of inbraakwerendheidsklasse wanden?</t>
+        </is>
+      </c>
+      <c r="C8" s="37" t="inlineStr">
+        <is>
+          <t>Niet in dit document</t>
+        </is>
+      </c>
+      <c r="D8" s="37" t="inlineStr">
+        <is>
+          <t>Geen extra klasse meegeprijsd.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="37" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="37" t="inlineStr">
+        <is>
+          <t>59 dB: DnT,A of Rw? Vraagt dubbele frames 155–170 mm</t>
+        </is>
+      </c>
+      <c r="C9" s="37" t="inlineStr">
+        <is>
+          <t>Niet in dit document</t>
+        </is>
+      </c>
+      <c r="D9" s="37" t="inlineStr">
+        <is>
+          <t>Dubbele frame wand meegeprijsd voor kantoor/gespreksruimten (60 m²).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="37" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="37" t="inlineStr">
+        <is>
+          <t>Alle kamerscheidende wanden volledig nieuw, plafond eruit</t>
+        </is>
+      </c>
+      <c r="C10" s="37" t="inlineStr">
+        <is>
+          <t>Niet in dit document</t>
+        </is>
+      </c>
+      <c r="D10" s="37" t="inlineStr">
+        <is>
+          <t>Zo meegeprijsd: 300 m1 nieuwe wand tot betondek.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="37" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="37" t="inlineStr">
+        <is>
+          <t>Brandklasse gordijnen en tapijt?</t>
+        </is>
+      </c>
+      <c r="C11" s="37" t="inlineStr">
+        <is>
+          <t>Niet in dit document</t>
+        </is>
+      </c>
+      <c r="D11" s="37" t="inlineStr">
+        <is>
+          <t>Standaard brandklasse (Cfl-s1 / B1) in richtprijs; controleren.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="37" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="37" t="inlineStr">
+        <is>
+          <t>Planning krap: gunning 12 okt, start 9 nov, V&amp;G 4 weken vooraf</t>
+        </is>
+      </c>
+      <c r="C12" s="37" t="inlineStr">
+        <is>
+          <t>Niet in dit document</t>
+        </is>
+      </c>
+      <c r="D12" s="37" t="inlineStr">
+        <is>
+          <t>Versnellingsrisico verhoogd naar 70% × € 15.000.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="37" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="37" t="inlineStr">
+        <is>
+          <t>Betaald parkeren: regie, plek of kaart?</t>
+        </is>
+      </c>
+      <c r="C13" s="37" t="inlineStr">
+        <is>
+          <t>Niet in dit document</t>
+        </is>
+      </c>
+      <c r="D13" s="37" t="inlineStr">
+        <is>
+          <t>Parkeerkosten opgenomen in ABK (€ 1.800).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="37" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="37" t="inlineStr">
+        <is>
+          <t>Type systeemplafond of standaard 60x60 wit?</t>
+        </is>
+      </c>
+      <c r="C14" s="37" t="inlineStr">
+        <is>
+          <t>Niet in dit document</t>
+        </is>
+      </c>
+      <c r="D14" s="37" t="inlineStr">
+        <is>
+          <t>Standaard 600x600 wit aangehouden.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="37" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="37" t="inlineStr">
+        <is>
+          <t>Naadloos marmoleum i.p.v. tapijt/marmoleum per kamer?</t>
+        </is>
+      </c>
+      <c r="C15" s="37" t="inlineStr">
+        <is>
+          <t>Niet in dit document</t>
+        </is>
+      </c>
+      <c r="D15" s="37" t="inlineStr">
+        <is>
+          <t>Basis volgens bestek; genoemd als optimalisatie.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="37" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="37" t="inlineStr">
+        <is>
+          <t>RVS-kasten in keuken (64 personen) i.p.v. HPL?</t>
+        </is>
+      </c>
+      <c r="C16" s="37" t="inlineStr">
+        <is>
+          <t>Niet in dit document</t>
+        </is>
+      </c>
+      <c r="D16" s="37" t="inlineStr">
+        <is>
+          <t>Basis HPL volgens bestek; RVS als optimalisatie met meerprijs.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="37" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="37" t="inlineStr">
+        <is>
+          <t>Meubilair en inrichting door aannemer?</t>
+        </is>
+      </c>
+      <c r="C17" s="37" t="inlineStr">
+        <is>
+          <t>Niet in dit document</t>
+        </is>
+      </c>
+      <c r="D17" s="37" t="inlineStr">
+        <is>
+          <t>Niet meegeprijsd (niet in scope BBN).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="37" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="37" t="inlineStr">
+        <is>
+          <t>HPL-douchecabines zoals boven i.p.v. metal-stud + tegels?</t>
+        </is>
+      </c>
+      <c r="C18" s="37" t="inlineStr">
+        <is>
+          <t>Niet in dit document</t>
+        </is>
+      </c>
+      <c r="D18" s="37" t="inlineStr">
+        <is>
+          <t>Basis volgens bestek; HPL-cabines als optimalisatie.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="37" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="37" t="inlineStr">
+        <is>
+          <t>08:00–16:00 hard of afbouw een uur eerder/later?</t>
+        </is>
+      </c>
+      <c r="C19" s="37" t="inlineStr">
+        <is>
+          <t>Niet in dit document</t>
+        </is>
+      </c>
+      <c r="D19" s="37" t="inlineStr">
+        <is>
+          <t>Uitgegaan van 08:00–16:00 voor lawaaiig werk.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20"/>
+    <row r="21" ht="30" customHeight="1">
+      <c r="A21" s="35" t="inlineStr">
+        <is>
+          <t>Opvallend: de NvI noemt Gemeente Wijdemeren als aanbestedende dienst en is gedateerd na de oorspronkelijke sluitingsdatum (18-09). Controleer de actuele sluitingsdatum op TenderNed.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Tellingen uit de tekeningen (versie 2)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2"/>
+    <row r="3">
+      <c r="A3" s="33" t="inlineStr">
+        <is>
+          <t>Onderdeel</t>
+        </is>
+      </c>
+      <c r="B3" s="33" t="inlineStr">
+        <is>
+          <t>Aantal</t>
+        </is>
+      </c>
+      <c r="C3" s="33" t="inlineStr">
+        <is>
+          <t>Tekening</t>
+        </is>
+      </c>
+      <c r="D3" s="33" t="inlineStr">
+        <is>
+          <t>Toelichting</t>
+        </is>
+      </c>
+      <c r="E3" s="33" t="inlineStr">
+        <is>
+          <t>Zekerheid</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="37" t="inlineStr">
+        <is>
+          <t>Bewonerskamers</t>
+        </is>
+      </c>
+      <c r="B4" s="37" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="C4" s="37" t="inlineStr">
+        <is>
+          <t>L.0.01-A/B, E.001</t>
+        </is>
+      </c>
+      <c r="D4" s="37" t="inlineStr">
+        <is>
+          <t>17 in deel A (0.07–0.23), 12 in deel B (0.49–0.56, 0.50a, 0.74–0.76)</t>
+        </is>
+      </c>
+      <c r="E4" s="37" t="inlineStr">
+        <is>
+          <t>Hoog</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="37" t="inlineStr">
+        <is>
+          <t>Fancoils benodigd</t>
+        </is>
+      </c>
+      <c r="B5" s="37" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="C5" s="37" t="inlineStr">
+        <is>
+          <t>L.0.01-A/B</t>
+        </is>
+      </c>
+      <c r="D5" s="37" t="inlineStr">
+        <is>
+          <t>1 per kamer (29) + 3 keuken 0.24 + 1 keuken 0.64 + 1 personeelsruimte 0.73</t>
+        </is>
+      </c>
+      <c r="E5" s="37" t="inlineStr">
+        <is>
+          <t>Middel</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="37" t="inlineStr">
+        <is>
+          <t>Fancoils bestaand (demontage)</t>
+        </is>
+      </c>
+      <c r="B6" s="37" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="C6" s="37" t="inlineStr">
+        <is>
+          <t>D.0.01-A/B</t>
+        </is>
+      </c>
+      <c r="D6" s="37" t="inlineStr">
+        <is>
+          <t>19 in deel A, 10 in deel B</t>
+        </is>
+      </c>
+      <c r="E6" s="37" t="inlineStr">
+        <is>
+          <t>Middel</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="37" t="inlineStr">
+        <is>
+          <t>Kanaalverwarmers/-koelers</t>
+        </is>
+      </c>
+      <c r="B7" s="37" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C7" s="37" t="inlineStr">
+        <is>
+          <t>E&amp;W 7.1, L.0.01</t>
+        </is>
+      </c>
+      <c r="D7" s="37" t="inlineStr">
+        <is>
+          <t>0.04, 0.05, 0.44, 0.45, 0.62, 0.63</t>
+        </is>
+      </c>
+      <c r="E7" s="37" t="inlineStr">
+        <is>
+          <t>Middel</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="37" t="inlineStr">
+        <is>
+          <t>Brandkleppen</t>
+        </is>
+      </c>
+      <c r="B8" s="37" t="inlineStr">
+        <is>
+          <t>ca. 64</t>
+        </is>
+      </c>
+      <c r="C8" s="37" t="inlineStr">
+        <is>
+          <t>L.0.01, E.001</t>
+        </is>
+      </c>
+      <c r="D8" s="37" t="inlineStr">
+        <is>
+          <t>2 per kamer + ca. 6 in 60-min scheidingen</t>
+        </is>
+      </c>
+      <c r="E8" s="37" t="inlineStr">
+        <is>
+          <t>Middel</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="37" t="inlineStr">
+        <is>
+          <t>Roosters</t>
+        </is>
+      </c>
+      <c r="B9" s="37" t="inlineStr">
+        <is>
+          <t>ca. 230</t>
+        </is>
+      </c>
+      <c r="C9" s="37" t="inlineStr">
+        <is>
+          <t>L.0.01-A/B</t>
+        </is>
+      </c>
+      <c r="D9" s="37" t="inlineStr">
+        <is>
+          <t>6 per kamer + keukens/overige ruimten</t>
+        </is>
+      </c>
+      <c r="E9" s="37" t="inlineStr">
+        <is>
+          <t>Laag</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="37" t="inlineStr">
+        <is>
+          <t>Douches</t>
+        </is>
+      </c>
+      <c r="B10" s="37" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="C10" s="37" t="inlineStr">
+        <is>
+          <t>T.0.01</t>
+        </is>
+      </c>
+      <c r="D10" s="37" t="inlineStr">
+        <is>
+          <t>4 in 0.42, 4 in 0.37, 2 in 0.70/0.71</t>
+        </is>
+      </c>
+      <c r="E10" s="37" t="inlineStr">
+        <is>
+          <t>Hoog</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="37" t="inlineStr">
+        <is>
+          <t>Wastafels</t>
+        </is>
+      </c>
+      <c r="B11" s="37" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C11" s="37" t="inlineStr">
+        <is>
+          <t>T.0.01</t>
+        </is>
+      </c>
+      <c r="D11" s="37" t="inlineStr">
+        <is>
+          <t>4 in 0.42, 4 in 0.37</t>
+        </is>
+      </c>
+      <c r="E11" s="37" t="inlineStr">
+        <is>
+          <t>Hoog</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="37" t="inlineStr">
+        <is>
+          <t>Tappunten aanrecht</t>
+        </is>
+      </c>
+      <c r="B12" s="37" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C12" s="37" t="inlineStr">
+        <is>
+          <t>T.0.01</t>
+        </is>
+      </c>
+      <c r="D12" s="37" t="inlineStr">
+        <is>
+          <t>3 in 0.24, 3 in 0.64, 1 pantry 0.01</t>
+        </is>
+      </c>
+      <c r="E12" s="37" t="inlineStr">
+        <is>
+          <t>Middel</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="37" t="inlineStr">
+        <is>
+          <t>Wasmachines / drogers</t>
+        </is>
+      </c>
+      <c r="B13" s="37" t="inlineStr">
+        <is>
+          <t>4 / 3</t>
+        </is>
+      </c>
+      <c r="C13" s="37" t="inlineStr">
+        <is>
+          <t>T.0.01, E.001</t>
+        </is>
+      </c>
+      <c r="D13" s="37" t="inlineStr">
+        <is>
+          <t>wm/wd in 0.57</t>
+        </is>
+      </c>
+      <c r="E13" s="37" t="inlineStr">
+        <is>
+          <t>Hoog</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="37" t="inlineStr">
+        <is>
+          <t>Water naar kamers (pantry)</t>
+        </is>
+      </c>
+      <c r="B14" s="37" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="C14" s="37" t="inlineStr">
+        <is>
+          <t>T.0.01, R.0.01</t>
+        </is>
+      </c>
+      <c r="D14" s="37" t="inlineStr">
+        <is>
+          <t>Alleen koelkast (kk) per kamer</t>
+        </is>
+      </c>
+      <c r="E14" s="37" t="inlineStr">
+        <is>
+          <t>Hoog</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="37" t="inlineStr">
+        <is>
+          <t>Nieuwe VWA kelder</t>
+        </is>
+      </c>
+      <c r="B15" s="37" t="inlineStr">
+        <is>
+          <t>ca. 40 m</t>
+        </is>
+      </c>
+      <c r="C15" s="37" t="inlineStr">
+        <is>
+          <t>R.-1.01</t>
+        </is>
+      </c>
+      <c r="D15" s="37" t="inlineStr">
+        <is>
+          <t>Van keuken/badruimten naar vetafscheider</t>
+        </is>
+      </c>
+      <c r="E15" s="37" t="inlineStr">
+        <is>
+          <t>Laag</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="37" t="inlineStr">
+        <is>
+          <t>Armaturen</t>
+        </is>
+      </c>
+      <c r="B16" s="37" t="inlineStr">
+        <is>
+          <t>ca. 215</t>
+        </is>
+      </c>
+      <c r="C16" s="37" t="inlineStr">
+        <is>
+          <t>E.001</t>
+        </is>
+      </c>
+      <c r="D16" s="37" t="inlineStr">
+        <is>
+          <t>A1 92, E1 16, E2 20, F 8, W 9, H + typische kamers doorgerekend</t>
+        </is>
+      </c>
+      <c r="E16" s="37" t="inlineStr">
+        <is>
+          <t>Laag</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="37" t="inlineStr">
+        <is>
+          <t>Noodverlichting</t>
+        </is>
+      </c>
+      <c r="B17" s="37" t="inlineStr">
+        <is>
+          <t>ca. 25</t>
+        </is>
+      </c>
+      <c r="C17" s="37" t="inlineStr">
+        <is>
+          <t>E.001</t>
+        </is>
+      </c>
+      <c r="D17" s="37" t="inlineStr">
+        <is>
+          <t>11 NV/NV1-punten + pictogrammen</t>
+        </is>
+      </c>
+      <c r="E17" s="37" t="inlineStr">
+        <is>
+          <t>Laag</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="37" t="inlineStr">
+        <is>
+          <t>Wandcontactdozen</t>
+        </is>
+      </c>
+      <c r="B18" s="37" t="inlineStr">
+        <is>
+          <t>ca. 95</t>
+        </is>
+      </c>
+      <c r="C18" s="37" t="inlineStr">
+        <is>
+          <t>E.001</t>
+        </is>
+      </c>
+      <c r="D18" s="37" t="inlineStr">
+        <is>
+          <t>KK, 3O, Alg., WM, DR</t>
+        </is>
+      </c>
+      <c r="E18" s="37" t="inlineStr">
+        <is>
+          <t>Laag</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="37" t="inlineStr">
+        <is>
+          <t>Kooktoestel / afzuigkap-aansluitingen</t>
+        </is>
+      </c>
+      <c r="B19" s="37" t="inlineStr">
+        <is>
+          <t>7 / 7</t>
+        </is>
+      </c>
+      <c r="C19" s="37" t="inlineStr">
+        <is>
+          <t>E.001</t>
+        </is>
+      </c>
+      <c r="D19" s="37" t="inlineStr">
+        <is>
+          <t>KT en AK</t>
+        </is>
+      </c>
+      <c r="E19" s="37" t="inlineStr">
+        <is>
+          <t>Hoog</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="37" t="inlineStr">
+        <is>
+          <t>Data / Wi-Fi</t>
+        </is>
+      </c>
+      <c r="B20" s="37" t="inlineStr">
+        <is>
+          <t>8 / 12</t>
+        </is>
+      </c>
+      <c r="C20" s="37" t="inlineStr">
+        <is>
+          <t>E.001</t>
+        </is>
+      </c>
+      <c r="D20" s="37" t="inlineStr">
+        <is>
+          <t>D en Wi-Fi-codes</t>
+        </is>
+      </c>
+      <c r="E20" s="37" t="inlineStr">
+        <is>
+          <t>Hoog</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="37" t="inlineStr">
+        <is>
+          <t>BMI: handmelders / sirenes / automatische melders</t>
+        </is>
+      </c>
+      <c r="B21" s="37" t="inlineStr">
+        <is>
+          <t>4 / ca. 35 / ca. 24</t>
+        </is>
+      </c>
+      <c r="C21" s="37" t="inlineStr">
+        <is>
+          <t>E.001</t>
+        </is>
+      </c>
+      <c r="D21" s="37" t="inlineStr">
+        <is>
+          <t>HBM; SW-combinaties; R en R/SW</t>
+        </is>
+      </c>
+      <c r="E21" s="37" t="inlineStr">
+        <is>
+          <t>Middel</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="37" t="inlineStr">
+        <is>
+          <t>Kaartlezers / elektrische sluitplaten</t>
+        </is>
+      </c>
+      <c r="B22" s="37" t="inlineStr">
+        <is>
+          <t>3 / 2</t>
+        </is>
+      </c>
+      <c r="C22" s="37" t="inlineStr">
+        <is>
+          <t>E.001</t>
+        </is>
+      </c>
+      <c r="D22" s="37" t="inlineStr">
+        <is>
+          <t>Wijkt af van BBN 3.4.2 (ES per kamerdeur)</t>
+        </is>
+      </c>
+      <c r="E22" s="37" t="inlineStr">
+        <is>
+          <t>Hoog</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="37" t="inlineStr">
+        <is>
+          <t>Nieuwe binnenwanden</t>
+        </is>
+      </c>
+      <c r="B23" s="37" t="inlineStr">
+        <is>
+          <t>ca. 300 m1</t>
+        </is>
+      </c>
+      <c r="C23" s="37" t="inlineStr">
+        <is>
+          <t>Afgeleid uit stramien 7,2 m</t>
+        </is>
+      </c>
+      <c r="D23" s="37" t="inlineStr">
+        <is>
+          <t>Kamers 3,6 m breed; bouwkundige tekeningen ontbreken</t>
+        </is>
+      </c>
+      <c r="E23" s="37" t="inlineStr">
+        <is>
+          <t>Laag</t>
         </is>
       </c>
     </row>

</xml_diff>